<commit_message>
Refresh ESPN and Yahoo rankings
</commit_message>
<xml_diff>
--- a/frontend/public/data/2026/espn/merged_formatted.xlsx
+++ b/frontend/public/data/2026/espn/merged_formatted.xlsx
@@ -608,7 +608,7 @@
         <v>56</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -640,7 +640,7 @@
         <v>55</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -1280,7 +1280,7 @@
         <v>23</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -1312,7 +1312,7 @@
         <v>37</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26">
@@ -1696,7 +1696,7 @@
         <v>24</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38">
@@ -1728,7 +1728,7 @@
         <v>29</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39">
@@ -2272,7 +2272,7 @@
         <v>10</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56">
@@ -2368,7 +2368,7 @@
         <v>8</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59">
@@ -2432,7 +2432,7 @@
         <v>9</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="61">
@@ -2464,7 +2464,7 @@
         <v>9</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62">
@@ -2496,7 +2496,7 @@
         <v>6</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="63">
@@ -2528,7 +2528,7 @@
         <v>12</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="64">
@@ -2560,7 +2560,7 @@
         <v>10</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="65">
@@ -2592,7 +2592,7 @@
         <v>6</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="66">
@@ -2624,7 +2624,7 @@
         <v>5</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="67">
@@ -2656,7 +2656,7 @@
         <v>2</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="68">
@@ -2688,7 +2688,7 @@
         <v>2</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="69">
@@ -2720,7 +2720,7 @@
         <v>4</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="70">
@@ -2752,7 +2752,7 @@
         <v>6</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71">
@@ -2784,7 +2784,7 @@
         <v>4</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="72">
@@ -2816,7 +2816,7 @@
         <v>5</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="73">
@@ -2848,7 +2848,7 @@
         <v>3</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="74">
@@ -2880,7 +2880,7 @@
         <v>4</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="75">
@@ -2912,7 +2912,7 @@
         <v>10</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="76">
@@ -2944,7 +2944,7 @@
         <v>2</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="77">
@@ -2976,7 +2976,7 @@
         <v>4</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="78">
@@ -3008,7 +3008,7 @@
         <v>15</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="79">
@@ -3072,7 +3072,7 @@
         <v>13</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81">
@@ -3104,7 +3104,7 @@
         <v>8</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="82">
@@ -3136,7 +3136,7 @@
         <v>1</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="83">
@@ -3168,7 +3168,7 @@
         <v>4</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="84">
@@ -3200,7 +3200,7 @@
         <v>5</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="85">
@@ -3232,7 +3232,7 @@
         <v>2</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="86">
@@ -3264,7 +3264,7 @@
         <v>2</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="87">
@@ -3296,7 +3296,7 @@
         <v>2</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="88">
@@ -3360,7 +3360,7 @@
         <v>1</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="90">
@@ -3392,7 +3392,7 @@
         <v>4</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="91">
@@ -3424,7 +3424,7 @@
         <v>2</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
     </row>
     <row r="92">
@@ -3456,7 +3456,7 @@
         <v>3</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="93">
@@ -3488,7 +3488,7 @@
         <v>4</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="94">
@@ -3520,7 +3520,7 @@
         <v>5</v>
       </c>
       <c r="H94" s="3" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="95">
@@ -3552,7 +3552,7 @@
         <v>2</v>
       </c>
       <c r="H95" s="3" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="96">
@@ -3584,7 +3584,7 @@
         <v>7</v>
       </c>
       <c r="H96" s="3" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="97">
@@ -3616,7 +3616,7 @@
         <v>7</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="98">
@@ -3648,7 +3648,7 @@
         <v>3</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="99">
@@ -3680,7 +3680,7 @@
         <v>7</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="100">
@@ -3712,7 +3712,7 @@
         <v>1</v>
       </c>
       <c r="H100" s="3" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="101">
@@ -3744,7 +3744,7 @@
         <v>1</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>97</v>
+        <v>115</v>
       </c>
     </row>
     <row r="102">
@@ -3776,7 +3776,7 @@
         <v>1</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>98</v>
+        <v>116</v>
       </c>
     </row>
     <row r="103">
@@ -3808,7 +3808,7 @@
         <v>2</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="104">
@@ -3840,7 +3840,7 @@
         <v>1</v>
       </c>
       <c r="H104" s="3" t="n">
-        <v>103</v>
+        <v>110</v>
       </c>
     </row>
     <row r="105">
@@ -3872,7 +3872,7 @@
         <v>1</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="106">
@@ -3904,7 +3904,7 @@
         <v>3</v>
       </c>
       <c r="H106" s="3" t="n">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="107">
@@ -3936,7 +3936,7 @@
         <v>3</v>
       </c>
       <c r="H107" s="3" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
     </row>
     <row r="108">
@@ -3968,7 +3968,7 @@
         <v>2</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>119</v>
+        <v>107</v>
       </c>
     </row>
     <row r="109">
@@ -4000,7 +4000,7 @@
         <v>3</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>113</v>
+        <v>103</v>
       </c>
     </row>
     <row r="110">
@@ -4032,7 +4032,7 @@
         <v>2</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="111">
@@ -4064,7 +4064,7 @@
         <v>4</v>
       </c>
       <c r="H111" s="3" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
     </row>
     <row r="112">
@@ -4096,7 +4096,7 @@
         <v>0</v>
       </c>
       <c r="H112" s="3" t="n">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="113">
@@ -4128,7 +4128,7 @@
         <v>1</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="114">
@@ -4160,7 +4160,7 @@
         <v>2</v>
       </c>
       <c r="H114" s="3" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="115">
@@ -4192,7 +4192,7 @@
         <v>3</v>
       </c>
       <c r="H115" s="3" t="n">
-        <v>117</v>
+        <v>101</v>
       </c>
     </row>
     <row r="116">
@@ -4224,7 +4224,7 @@
         <v>1</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="117">
@@ -4256,7 +4256,7 @@
         <v>0</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="118">
@@ -4288,7 +4288,7 @@
         <v>2</v>
       </c>
       <c r="H118" s="3" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="119">
@@ -4320,7 +4320,7 @@
         <v>2</v>
       </c>
       <c r="H119" s="3" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="120">
@@ -4352,7 +4352,7 @@
         <v>0</v>
       </c>
       <c r="H120" s="3" t="n">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="121">
@@ -4384,7 +4384,7 @@
         <v>1</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="122">
@@ -4416,7 +4416,7 @@
         <v>3</v>
       </c>
       <c r="H122" s="3" t="n">
-        <v>158</v>
+        <v>121</v>
       </c>
     </row>
     <row r="123">
@@ -4448,7 +4448,7 @@
         <v>1</v>
       </c>
       <c r="H123" s="3" t="n">
-        <v>125</v>
+        <v>158</v>
       </c>
     </row>
     <row r="124">
@@ -4480,7 +4480,7 @@
         <v>2</v>
       </c>
       <c r="H124" s="3" t="n">
-        <v>156</v>
+        <v>125</v>
       </c>
     </row>
     <row r="125">
@@ -4512,7 +4512,7 @@
         <v>1</v>
       </c>
       <c r="H125" s="3" t="n">
-        <v>157</v>
+        <v>126</v>
       </c>
     </row>
     <row r="126">
@@ -4544,7 +4544,7 @@
         <v>2</v>
       </c>
       <c r="H126" s="3" t="n">
-        <v>145</v>
+        <v>124</v>
       </c>
     </row>
     <row r="127">
@@ -4576,7 +4576,7 @@
         <v>3</v>
       </c>
       <c r="H127" s="3" t="n">
-        <v>147</v>
+        <v>122</v>
       </c>
     </row>
     <row r="128">
@@ -4608,7 +4608,7 @@
         <v>1</v>
       </c>
       <c r="H128" s="3" t="n">
-        <v>155</v>
+        <v>139</v>
       </c>
     </row>
     <row r="129">
@@ -4640,7 +4640,7 @@
         <v>4</v>
       </c>
       <c r="H129" s="3" t="n">
-        <v>150</v>
+        <v>127</v>
       </c>
     </row>
     <row r="130">
@@ -4672,7 +4672,7 @@
         <v>1</v>
       </c>
       <c r="H130" s="3" t="n">
-        <v>151</v>
+        <v>135</v>
       </c>
     </row>
     <row r="131">
@@ -4704,7 +4704,7 @@
         <v>0</v>
       </c>
       <c r="H131" s="3" t="n">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="132">
@@ -4736,7 +4736,7 @@
         <v>1</v>
       </c>
       <c r="H132" s="3" t="n">
-        <v>153</v>
+        <v>142</v>
       </c>
     </row>
     <row r="133">
@@ -4768,7 +4768,7 @@
         <v>1</v>
       </c>
       <c r="H133" s="3" t="n">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="134">
@@ -4800,7 +4800,7 @@
         <v>2</v>
       </c>
       <c r="H134" s="3" t="n">
-        <v>159</v>
+        <v>137</v>
       </c>
     </row>
     <row r="135">
@@ -4832,7 +4832,7 @@
         <v>0</v>
       </c>
       <c r="H135" s="3" t="n">
-        <v>121</v>
+        <v>146</v>
       </c>
     </row>
     <row r="136">
@@ -4864,7 +4864,7 @@
         <v>0</v>
       </c>
       <c r="H136" s="3" t="n">
-        <v>124</v>
+        <v>153</v>
       </c>
     </row>
     <row r="137">
@@ -4896,7 +4896,7 @@
         <v>2</v>
       </c>
       <c r="H137" s="3" t="n">
-        <v>149</v>
+        <v>136</v>
       </c>
     </row>
     <row r="138">
@@ -4928,7 +4928,7 @@
         <v>0</v>
       </c>
       <c r="H138" s="3" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="139">
@@ -4960,7 +4960,7 @@
         <v>0</v>
       </c>
       <c r="H139" s="3" t="n">
-        <v>127</v>
+        <v>147</v>
       </c>
     </row>
     <row r="140">
@@ -4992,7 +4992,7 @@
         <v>0</v>
       </c>
       <c r="H140" s="3" t="n">
-        <v>123</v>
+        <v>144</v>
       </c>
     </row>
     <row r="141">
@@ -5024,7 +5024,7 @@
         <v>2</v>
       </c>
       <c r="H141" s="3" t="n">
-        <v>154</v>
+        <v>123</v>
       </c>
     </row>
     <row r="142">
@@ -5056,7 +5056,7 @@
         <v>0</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>133</v>
+        <v>155</v>
       </c>
     </row>
     <row r="143">
@@ -5088,7 +5088,7 @@
         <v>0</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>122</v>
+        <v>141</v>
       </c>
     </row>
     <row r="144">
@@ -5120,7 +5120,7 @@
         <v>0</v>
       </c>
       <c r="H144" s="3" t="n">
-        <v>132</v>
+        <v>148</v>
       </c>
     </row>
     <row r="145">
@@ -5152,7 +5152,7 @@
         <v>0</v>
       </c>
       <c r="H145" s="3" t="n">
-        <v>143</v>
+        <v>150</v>
       </c>
     </row>
     <row r="146">
@@ -5184,7 +5184,7 @@
         <v>0</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
     </row>
     <row r="147">
@@ -5216,7 +5216,7 @@
         <v>1</v>
       </c>
       <c r="H147" s="3" t="n">
-        <v>160</v>
+        <v>138</v>
       </c>
     </row>
     <row r="148">
@@ -5248,7 +5248,7 @@
         <v>0</v>
       </c>
       <c r="H148" s="3" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="149">
@@ -5280,7 +5280,7 @@
         <v>0</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>142</v>
+        <v>131</v>
       </c>
     </row>
     <row r="150">
@@ -5312,7 +5312,7 @@
         <v>2</v>
       </c>
       <c r="H150" s="3" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
     </row>
     <row r="151">
@@ -5344,7 +5344,7 @@
         <v>1</v>
       </c>
       <c r="H151" s="3" t="n">
-        <v>144</v>
+        <v>159</v>
       </c>
     </row>
     <row r="152">
@@ -5376,7 +5376,7 @@
         <v>0</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>130</v>
+        <v>157</v>
       </c>
     </row>
     <row r="153">
@@ -5408,7 +5408,7 @@
         <v>0</v>
       </c>
       <c r="H153" s="3" t="n">
-        <v>131</v>
+        <v>152</v>
       </c>
     </row>
     <row r="154">
@@ -5440,7 +5440,7 @@
         <v>0</v>
       </c>
       <c r="H154" s="3" t="n">
-        <v>136</v>
+        <v>151</v>
       </c>
     </row>
     <row r="155">
@@ -5472,7 +5472,7 @@
         <v>0</v>
       </c>
       <c r="H155" s="3" t="n">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="156">
@@ -5504,7 +5504,7 @@
         <v>0</v>
       </c>
       <c r="H156" s="3" t="n">
-        <v>137</v>
+        <v>160</v>
       </c>
     </row>
     <row r="157">
@@ -5536,7 +5536,7 @@
         <v>1</v>
       </c>
       <c r="H157" s="3" t="n">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="158">
@@ -5568,7 +5568,7 @@
         <v>0</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>126</v>
+        <v>145</v>
       </c>
     </row>
     <row r="159">
@@ -5600,7 +5600,7 @@
         <v>1</v>
       </c>
       <c r="H159" s="3" t="n">
-        <v>128</v>
+        <v>156</v>
       </c>
     </row>
     <row r="160">
@@ -5632,7 +5632,7 @@
         <v>0</v>
       </c>
       <c r="H160" s="3" t="n">
-        <v>141</v>
+        <v>129</v>
       </c>
     </row>
     <row r="161">
@@ -5664,7 +5664,7 @@
         <v>0</v>
       </c>
       <c r="H161" s="3" t="n">
-        <v>134</v>
+        <v>154</v>
       </c>
     </row>
     <row r="162">
@@ -5696,7 +5696,7 @@
         <v>1</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>206</v>
+        <v>191</v>
       </c>
     </row>
     <row r="163">
@@ -5728,7 +5728,7 @@
         <v>0</v>
       </c>
       <c r="H163" s="3" t="n">
-        <v>196</v>
+        <v>240</v>
       </c>
     </row>
     <row r="164">
@@ -5760,7 +5760,7 @@
         <v>0</v>
       </c>
       <c r="H164" s="3" t="n">
-        <v>254</v>
+        <v>183</v>
       </c>
     </row>
     <row r="165">
@@ -5792,7 +5792,7 @@
         <v>0</v>
       </c>
       <c r="H165" s="3" t="n">
-        <v>195</v>
+        <v>241</v>
       </c>
     </row>
     <row r="166">
@@ -5824,7 +5824,7 @@
         <v>0</v>
       </c>
       <c r="H166" s="3" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="167">
@@ -5856,7 +5856,7 @@
         <v>0</v>
       </c>
       <c r="H167" s="3" t="n">
-        <v>221</v>
+        <v>168</v>
       </c>
     </row>
     <row r="168">
@@ -5888,7 +5888,7 @@
         <v>0</v>
       </c>
       <c r="H168" s="3" t="n">
-        <v>200</v>
+        <v>236</v>
       </c>
     </row>
     <row r="169">
@@ -5920,7 +5920,7 @@
         <v>1</v>
       </c>
       <c r="H169" s="3" t="n">
-        <v>208</v>
+        <v>163</v>
       </c>
     </row>
     <row r="170">
@@ -5952,7 +5952,7 @@
         <v>2</v>
       </c>
       <c r="H170" s="3" t="n">
-        <v>242</v>
+        <v>165</v>
       </c>
     </row>
     <row r="171">
@@ -5984,7 +5984,7 @@
         <v>1</v>
       </c>
       <c r="H171" s="3" t="n">
-        <v>214</v>
+        <v>161</v>
       </c>
     </row>
     <row r="172">
@@ -6016,7 +6016,7 @@
         <v>1</v>
       </c>
       <c r="H172" s="3" t="n">
-        <v>215</v>
+        <v>162</v>
       </c>
     </row>
     <row r="173">
@@ -6048,7 +6048,7 @@
         <v>0</v>
       </c>
       <c r="H173" s="3" t="n">
-        <v>233</v>
+        <v>182</v>
       </c>
     </row>
     <row r="174">
@@ -6080,7 +6080,7 @@
         <v>1</v>
       </c>
       <c r="H174" s="3" t="n">
-        <v>222</v>
+        <v>186</v>
       </c>
     </row>
     <row r="175">
@@ -6112,7 +6112,7 @@
         <v>0</v>
       </c>
       <c r="H175" s="3" t="n">
-        <v>227</v>
+        <v>173</v>
       </c>
     </row>
     <row r="176">
@@ -6144,7 +6144,7 @@
         <v>0</v>
       </c>
       <c r="H176" s="3" t="n">
-        <v>219</v>
+        <v>188</v>
       </c>
     </row>
     <row r="177">
@@ -6176,7 +6176,7 @@
         <v>1</v>
       </c>
       <c r="H177" s="3" t="n">
-        <v>211</v>
+        <v>166</v>
       </c>
     </row>
     <row r="178">
@@ -6208,7 +6208,7 @@
         <v>0</v>
       </c>
       <c r="H178" s="3" t="n">
-        <v>226</v>
+        <v>174</v>
       </c>
     </row>
     <row r="179">
@@ -6240,7 +6240,7 @@
         <v>1</v>
       </c>
       <c r="H179" s="3" t="n">
-        <v>229</v>
+        <v>171</v>
       </c>
     </row>
     <row r="180">
@@ -6272,7 +6272,7 @@
         <v>1</v>
       </c>
       <c r="H180" s="3" t="n">
-        <v>238</v>
+        <v>184</v>
       </c>
     </row>
     <row r="181">
@@ -6304,7 +6304,7 @@
         <v>0</v>
       </c>
       <c r="H181" s="3" t="n">
-        <v>218</v>
+        <v>189</v>
       </c>
     </row>
     <row r="182">
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="H182" s="3" t="n">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="183">
@@ -6368,7 +6368,7 @@
         <v>0</v>
       </c>
       <c r="H183" s="3" t="n">
-        <v>210</v>
+        <v>178</v>
       </c>
     </row>
     <row r="184">
@@ -6400,7 +6400,7 @@
         <v>0</v>
       </c>
       <c r="H184" s="3" t="n">
-        <v>203</v>
+        <v>233</v>
       </c>
     </row>
     <row r="185">
@@ -6432,7 +6432,7 @@
         <v>0</v>
       </c>
       <c r="H185" s="3" t="n">
-        <v>176</v>
+        <v>218</v>
       </c>
     </row>
     <row r="186">
@@ -6464,7 +6464,7 @@
         <v>0</v>
       </c>
       <c r="H186" s="3" t="n">
-        <v>177</v>
+        <v>219</v>
       </c>
     </row>
     <row r="187">
@@ -6496,7 +6496,7 @@
         <v>2</v>
       </c>
       <c r="H187" s="3" t="n">
-        <v>246</v>
+        <v>164</v>
       </c>
     </row>
     <row r="188">
@@ -6528,7 +6528,7 @@
         <v>0</v>
       </c>
       <c r="H188" s="3" t="n">
-        <v>251</v>
+        <v>198</v>
       </c>
     </row>
     <row r="189">
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="H189" s="3" t="n">
-        <v>225</v>
+        <v>167</v>
       </c>
     </row>
     <row r="190">
@@ -6592,7 +6592,7 @@
         <v>0</v>
       </c>
       <c r="H190" s="3" t="n">
-        <v>161</v>
+        <v>223</v>
       </c>
     </row>
     <row r="191">
@@ -6624,7 +6624,7 @@
         <v>0</v>
       </c>
       <c r="H191" s="3" t="n">
-        <v>253</v>
+        <v>180</v>
       </c>
     </row>
     <row r="192">
@@ -6656,7 +6656,7 @@
         <v>1</v>
       </c>
       <c r="H192" s="3" t="n">
-        <v>220</v>
+        <v>185</v>
       </c>
     </row>
     <row r="193">
@@ -6688,7 +6688,7 @@
         <v>0</v>
       </c>
       <c r="H193" s="3" t="n">
-        <v>249</v>
+        <v>196</v>
       </c>
     </row>
     <row r="194">
@@ -6720,7 +6720,7 @@
         <v>0</v>
       </c>
       <c r="H194" s="3" t="n">
-        <v>201</v>
+        <v>235</v>
       </c>
     </row>
     <row r="195">
@@ -6752,7 +6752,7 @@
         <v>0</v>
       </c>
       <c r="H195" s="3" t="n">
-        <v>244</v>
+        <v>192</v>
       </c>
     </row>
     <row r="196">
@@ -6784,7 +6784,7 @@
         <v>0</v>
       </c>
       <c r="H196" s="3" t="n">
-        <v>252</v>
+        <v>197</v>
       </c>
     </row>
     <row r="197">
@@ -6816,7 +6816,7 @@
         <v>0</v>
       </c>
       <c r="H197" s="3" t="n">
-        <v>232</v>
+        <v>209</v>
       </c>
     </row>
     <row r="198">
@@ -6848,7 +6848,7 @@
         <v>0</v>
       </c>
       <c r="H198" s="3" t="n">
-        <v>234</v>
+        <v>205</v>
       </c>
     </row>
     <row r="199">
@@ -6880,7 +6880,7 @@
         <v>0</v>
       </c>
       <c r="H199" s="3" t="n">
-        <v>191</v>
+        <v>245</v>
       </c>
     </row>
     <row r="200">
@@ -6912,7 +6912,7 @@
         <v>0</v>
       </c>
       <c r="H200" s="3" t="n">
-        <v>235</v>
+        <v>204</v>
       </c>
     </row>
     <row r="201">
@@ -6944,7 +6944,7 @@
         <v>0</v>
       </c>
       <c r="H201" s="3" t="n">
-        <v>183</v>
+        <v>253</v>
       </c>
     </row>
     <row r="202">
@@ -6976,7 +6976,7 @@
         <v>0</v>
       </c>
       <c r="H202" s="3" t="n">
-        <v>199</v>
+        <v>237</v>
       </c>
     </row>
     <row r="203">
@@ -7008,7 +7008,7 @@
         <v>0</v>
       </c>
       <c r="H203" s="3" t="n">
-        <v>164</v>
+        <v>215</v>
       </c>
     </row>
     <row r="204">
@@ -7040,7 +7040,7 @@
         <v>0</v>
       </c>
       <c r="H204" s="3" t="n">
-        <v>231</v>
+        <v>181</v>
       </c>
     </row>
     <row r="205">
@@ -7072,7 +7072,7 @@
         <v>0</v>
       </c>
       <c r="H205" s="3" t="n">
-        <v>223</v>
+        <v>169</v>
       </c>
     </row>
     <row r="206">
@@ -7104,7 +7104,7 @@
         <v>0</v>
       </c>
       <c r="H206" s="3" t="n">
-        <v>224</v>
+        <v>170</v>
       </c>
     </row>
     <row r="207">
@@ -7136,7 +7136,7 @@
         <v>0</v>
       </c>
       <c r="H207" s="3" t="n">
-        <v>216</v>
+        <v>175</v>
       </c>
     </row>
     <row r="208">
@@ -7168,7 +7168,7 @@
         <v>0</v>
       </c>
       <c r="H208" s="3" t="n">
-        <v>250</v>
+        <v>199</v>
       </c>
     </row>
     <row r="209">
@@ -7200,7 +7200,7 @@
         <v>0</v>
       </c>
       <c r="H209" s="3" t="n">
-        <v>236</v>
+        <v>202</v>
       </c>
     </row>
     <row r="210">
@@ -7264,7 +7264,7 @@
         <v>0</v>
       </c>
       <c r="H211" s="3" t="n">
-        <v>163</v>
+        <v>226</v>
       </c>
     </row>
     <row r="212">
@@ -7296,7 +7296,7 @@
         <v>0</v>
       </c>
       <c r="H212" s="3" t="n">
-        <v>168</v>
+        <v>224</v>
       </c>
     </row>
     <row r="213">
@@ -7328,7 +7328,7 @@
         <v>0</v>
       </c>
       <c r="H213" s="3" t="n">
-        <v>213</v>
+        <v>187</v>
       </c>
     </row>
     <row r="214">
@@ -7360,7 +7360,7 @@
         <v>0</v>
       </c>
       <c r="H214" s="3" t="n">
-        <v>186</v>
+        <v>250</v>
       </c>
     </row>
     <row r="215">
@@ -7392,7 +7392,7 @@
         <v>0</v>
       </c>
       <c r="H215" s="3" t="n">
-        <v>194</v>
+        <v>242</v>
       </c>
     </row>
     <row r="216">
@@ -7424,7 +7424,7 @@
         <v>0</v>
       </c>
       <c r="H216" s="3" t="n">
-        <v>178</v>
+        <v>213</v>
       </c>
     </row>
     <row r="217">
@@ -7456,7 +7456,7 @@
         <v>0</v>
       </c>
       <c r="H217" s="3" t="n">
-        <v>192</v>
+        <v>244</v>
       </c>
     </row>
     <row r="218">
@@ -7488,7 +7488,7 @@
         <v>0</v>
       </c>
       <c r="H218" s="3" t="n">
-        <v>180</v>
+        <v>229</v>
       </c>
     </row>
     <row r="219">
@@ -7520,7 +7520,7 @@
         <v>0</v>
       </c>
       <c r="H219" s="3" t="n">
-        <v>237</v>
+        <v>203</v>
       </c>
     </row>
     <row r="220">
@@ -7552,7 +7552,7 @@
         <v>0</v>
       </c>
       <c r="H220" s="3" t="n">
-        <v>217</v>
+        <v>190</v>
       </c>
     </row>
     <row r="221">
@@ -7584,7 +7584,7 @@
         <v>0</v>
       </c>
       <c r="H221" s="3" t="n">
-        <v>230</v>
+        <v>176</v>
       </c>
     </row>
     <row r="222">
@@ -7616,7 +7616,7 @@
         <v>0</v>
       </c>
       <c r="H222" s="3" t="n">
-        <v>190</v>
+        <v>246</v>
       </c>
     </row>
     <row r="223">
@@ -7648,7 +7648,7 @@
         <v>0</v>
       </c>
       <c r="H223" s="3" t="n">
-        <v>179</v>
+        <v>232</v>
       </c>
     </row>
     <row r="224">
@@ -7680,7 +7680,7 @@
         <v>0</v>
       </c>
       <c r="H224" s="3" t="n">
-        <v>243</v>
+        <v>206</v>
       </c>
     </row>
     <row r="225">
@@ -7712,7 +7712,7 @@
         <v>0</v>
       </c>
       <c r="H225" s="3" t="n">
-        <v>165</v>
+        <v>225</v>
       </c>
     </row>
     <row r="226">
@@ -7744,7 +7744,7 @@
         <v>0</v>
       </c>
       <c r="H226" s="3" t="n">
-        <v>174</v>
+        <v>220</v>
       </c>
     </row>
     <row r="227">
@@ -7776,7 +7776,7 @@
         <v>0</v>
       </c>
       <c r="H227" s="3" t="n">
-        <v>187</v>
+        <v>249</v>
       </c>
     </row>
     <row r="228">
@@ -7808,7 +7808,7 @@
         <v>0</v>
       </c>
       <c r="H228" s="3" t="n">
-        <v>167</v>
+        <v>212</v>
       </c>
     </row>
     <row r="229">
@@ -7840,7 +7840,7 @@
         <v>1</v>
       </c>
       <c r="H229" s="3" t="n">
-        <v>228</v>
+        <v>172</v>
       </c>
     </row>
     <row r="230">
@@ -7872,7 +7872,7 @@
         <v>0</v>
       </c>
       <c r="H230" s="3" t="n">
-        <v>240</v>
+        <v>201</v>
       </c>
     </row>
     <row r="231">
@@ -7904,7 +7904,7 @@
         <v>0</v>
       </c>
       <c r="H231" s="3" t="n">
-        <v>212</v>
+        <v>179</v>
       </c>
     </row>
     <row r="232">
@@ -7936,7 +7936,7 @@
         <v>0</v>
       </c>
       <c r="H232" s="3" t="n">
-        <v>245</v>
+        <v>193</v>
       </c>
     </row>
     <row r="233">
@@ -7968,7 +7968,7 @@
         <v>0</v>
       </c>
       <c r="H233" s="3" t="n">
-        <v>239</v>
+        <v>200</v>
       </c>
     </row>
     <row r="234">
@@ -8000,7 +8000,7 @@
         <v>0</v>
       </c>
       <c r="H234" s="3" t="n">
-        <v>189</v>
+        <v>247</v>
       </c>
     </row>
     <row r="235">
@@ -8032,7 +8032,7 @@
         <v>0</v>
       </c>
       <c r="H235" s="3" t="n">
-        <v>193</v>
+        <v>243</v>
       </c>
     </row>
     <row r="236">
@@ -8064,7 +8064,7 @@
         <v>0</v>
       </c>
       <c r="H236" s="3" t="n">
-        <v>182</v>
+        <v>254</v>
       </c>
     </row>
     <row r="237">
@@ -8096,7 +8096,7 @@
         <v>0</v>
       </c>
       <c r="H237" s="3" t="n">
-        <v>188</v>
+        <v>248</v>
       </c>
     </row>
     <row r="238">
@@ -8128,7 +8128,7 @@
         <v>0</v>
       </c>
       <c r="H238" s="3" t="n">
-        <v>185</v>
+        <v>251</v>
       </c>
     </row>
     <row r="239">
@@ -8160,7 +8160,7 @@
         <v>0</v>
       </c>
       <c r="H239" s="3" t="n">
-        <v>248</v>
+        <v>195</v>
       </c>
     </row>
     <row r="240">
@@ -8192,7 +8192,7 @@
         <v>0</v>
       </c>
       <c r="H240" s="3" t="n">
-        <v>241</v>
+        <v>207</v>
       </c>
     </row>
     <row r="241">
@@ -8224,7 +8224,7 @@
         <v>0</v>
       </c>
       <c r="H241" s="3" t="n">
-        <v>169</v>
+        <v>217</v>
       </c>
     </row>
     <row r="242">
@@ -8256,7 +8256,7 @@
         <v>0</v>
       </c>
       <c r="H242" s="3" t="n">
-        <v>171</v>
+        <v>216</v>
       </c>
     </row>
     <row r="243">
@@ -8288,7 +8288,7 @@
         <v>0</v>
       </c>
       <c r="H243" s="3" t="n">
-        <v>181</v>
+        <v>230</v>
       </c>
     </row>
     <row r="244">
@@ -8320,7 +8320,7 @@
         <v>0</v>
       </c>
       <c r="H244" s="3" t="n">
-        <v>170</v>
+        <v>222</v>
       </c>
     </row>
     <row r="245">
@@ -8352,7 +8352,7 @@
         <v>0</v>
       </c>
       <c r="H245" s="3" t="n">
-        <v>166</v>
+        <v>210</v>
       </c>
     </row>
     <row r="246">
@@ -8384,7 +8384,7 @@
         <v>0</v>
       </c>
       <c r="H246" s="3" t="n">
-        <v>197</v>
+        <v>239</v>
       </c>
     </row>
     <row r="247">
@@ -8416,7 +8416,7 @@
         <v>0</v>
       </c>
       <c r="H247" s="3" t="n">
-        <v>204</v>
+        <v>231</v>
       </c>
     </row>
     <row r="248">
@@ -8448,7 +8448,7 @@
         <v>0</v>
       </c>
       <c r="H248" s="3" t="n">
-        <v>173</v>
+        <v>214</v>
       </c>
     </row>
     <row r="249">
@@ -8480,7 +8480,7 @@
         <v>0</v>
       </c>
       <c r="H249" s="3" t="n">
-        <v>202</v>
+        <v>234</v>
       </c>
     </row>
     <row r="250">
@@ -8512,7 +8512,7 @@
         <v>0</v>
       </c>
       <c r="H250" s="3" t="n">
-        <v>247</v>
+        <v>194</v>
       </c>
     </row>
     <row r="251">
@@ -8544,7 +8544,7 @@
         <v>0</v>
       </c>
       <c r="H251" s="3" t="n">
-        <v>209</v>
+        <v>177</v>
       </c>
     </row>
     <row r="252">
@@ -8576,7 +8576,7 @@
         <v>0</v>
       </c>
       <c r="H252" s="3" t="n">
-        <v>175</v>
+        <v>228</v>
       </c>
     </row>
     <row r="253">
@@ -8608,7 +8608,7 @@
         <v>0</v>
       </c>
       <c r="H253" s="3" t="n">
-        <v>162</v>
+        <v>227</v>
       </c>
     </row>
     <row r="254">
@@ -8640,7 +8640,7 @@
         <v>0</v>
       </c>
       <c r="H254" s="3" t="n">
-        <v>198</v>
+        <v>238</v>
       </c>
     </row>
     <row r="255">
@@ -8672,7 +8672,7 @@
         <v>0</v>
       </c>
       <c r="H255" s="3" t="n">
-        <v>184</v>
+        <v>252</v>
       </c>
     </row>
     <row r="256">
@@ -8704,7 +8704,7 @@
         <v>0</v>
       </c>
       <c r="H256" s="3" t="n">
-        <v>172</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add selectable Yahoo PPR ranking profiles
</commit_message>
<xml_diff>
--- a/frontend/public/data/2026/espn/merged_formatted.xlsx
+++ b/frontend/public/data/2026/espn/merged_formatted.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H256"/>
+  <dimension ref="A1:I256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -546,6 +546,11 @@
           <t>PriceRank</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Adjusted Rank Half PPR</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -578,6 +583,9 @@
       <c r="H2" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I2" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -608,7 +616,10 @@
         <v>55</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -640,6 +651,9 @@
         <v>56</v>
       </c>
       <c r="H4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" s="3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -674,6 +688,9 @@
       <c r="H5" s="3" t="n">
         <v>4</v>
       </c>
+      <c r="I5" s="3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -706,6 +723,9 @@
       <c r="H6" s="3" t="n">
         <v>5</v>
       </c>
+      <c r="I6" s="3" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -738,6 +758,9 @@
       <c r="H7" s="3" t="n">
         <v>6</v>
       </c>
+      <c r="I7" s="3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -770,6 +793,9 @@
       <c r="H8" s="3" t="n">
         <v>7</v>
       </c>
+      <c r="I8" s="3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -802,6 +828,9 @@
       <c r="H9" s="3" t="n">
         <v>8</v>
       </c>
+      <c r="I9" s="3" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -834,6 +863,9 @@
       <c r="H10" s="3" t="n">
         <v>9</v>
       </c>
+      <c r="I10" s="3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -866,6 +898,9 @@
       <c r="H11" s="3" t="n">
         <v>10</v>
       </c>
+      <c r="I11" s="3" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -898,6 +933,9 @@
       <c r="H12" s="3" t="n">
         <v>11</v>
       </c>
+      <c r="I12" s="3" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -930,6 +968,9 @@
       <c r="H13" s="3" t="n">
         <v>12</v>
       </c>
+      <c r="I13" s="3" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -962,6 +1003,9 @@
       <c r="H14" s="3" t="n">
         <v>13</v>
       </c>
+      <c r="I14" s="3" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -994,6 +1038,9 @@
       <c r="H15" s="3" t="n">
         <v>14</v>
       </c>
+      <c r="I15" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1026,6 +1073,9 @@
       <c r="H16" s="3" t="n">
         <v>15</v>
       </c>
+      <c r="I16" s="3" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1058,6 +1108,9 @@
       <c r="H17" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="I17" s="3" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1090,6 +1143,9 @@
       <c r="H18" s="3" t="n">
         <v>17</v>
       </c>
+      <c r="I18" s="3" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1122,6 +1178,9 @@
       <c r="H19" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="I19" s="3" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1154,6 +1213,9 @@
       <c r="H20" s="3" t="n">
         <v>19</v>
       </c>
+      <c r="I20" s="3" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1186,6 +1248,9 @@
       <c r="H21" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="I21" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1218,6 +1283,9 @@
       <c r="H22" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="I22" s="3" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1250,6 +1318,9 @@
       <c r="H23" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="I23" s="3" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1282,6 +1353,9 @@
       <c r="H24" s="3" t="n">
         <v>24</v>
       </c>
+      <c r="I24" s="3" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1314,6 +1388,9 @@
       <c r="H25" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="I25" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1346,6 +1423,9 @@
       <c r="H26" s="3" t="n">
         <v>25</v>
       </c>
+      <c r="I26" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1378,6 +1458,9 @@
       <c r="H27" s="3" t="n">
         <v>26</v>
       </c>
+      <c r="I27" s="3" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1410,6 +1493,9 @@
       <c r="H28" s="3" t="n">
         <v>27</v>
       </c>
+      <c r="I28" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1442,6 +1528,9 @@
       <c r="H29" s="3" t="n">
         <v>28</v>
       </c>
+      <c r="I29" s="3" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -1474,6 +1563,9 @@
       <c r="H30" s="3" t="n">
         <v>29</v>
       </c>
+      <c r="I30" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1506,6 +1598,9 @@
       <c r="H31" s="3" t="n">
         <v>30</v>
       </c>
+      <c r="I31" s="3" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1538,6 +1633,9 @@
       <c r="H32" s="3" t="n">
         <v>31</v>
       </c>
+      <c r="I32" s="3" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -1570,6 +1668,9 @@
       <c r="H33" s="3" t="n">
         <v>32</v>
       </c>
+      <c r="I33" s="3" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -1602,6 +1703,9 @@
       <c r="H34" s="3" t="n">
         <v>33</v>
       </c>
+      <c r="I34" s="3" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -1634,6 +1738,9 @@
       <c r="H35" s="3" t="n">
         <v>34</v>
       </c>
+      <c r="I35" s="3" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1664,7 +1771,10 @@
         <v>30</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="37">
@@ -1698,6 +1808,9 @@
       <c r="H37" s="3" t="n">
         <v>35</v>
       </c>
+      <c r="I37" s="3" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1728,7 +1841,10 @@
         <v>24</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="39">
@@ -1762,6 +1878,9 @@
       <c r="H39" s="3" t="n">
         <v>39</v>
       </c>
+      <c r="I39" s="3" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1794,6 +1913,9 @@
       <c r="H40" s="3" t="n">
         <v>38</v>
       </c>
+      <c r="I40" s="3" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1826,6 +1948,9 @@
       <c r="H41" s="3" t="n">
         <v>40</v>
       </c>
+      <c r="I41" s="3" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1856,7 +1981,10 @@
         <v>6</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>69</v>
       </c>
     </row>
     <row r="43">
@@ -1888,7 +2016,10 @@
         <v>22</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="44">
@@ -1922,6 +2053,9 @@
       <c r="H44" s="3" t="n">
         <v>43</v>
       </c>
+      <c r="I44" s="3" t="n">
+        <v>54</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -1954,6 +2088,9 @@
       <c r="H45" s="3" t="n">
         <v>44</v>
       </c>
+      <c r="I45" s="3" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -1986,6 +2123,9 @@
       <c r="H46" s="3" t="n">
         <v>45</v>
       </c>
+      <c r="I46" s="3" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -2018,6 +2158,9 @@
       <c r="H47" s="3" t="n">
         <v>46</v>
       </c>
+      <c r="I47" s="3" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -2050,6 +2193,9 @@
       <c r="H48" s="3" t="n">
         <v>47</v>
       </c>
+      <c r="I48" s="3" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -2082,6 +2228,9 @@
       <c r="H49" s="3" t="n">
         <v>48</v>
       </c>
+      <c r="I49" s="3" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
@@ -2114,6 +2263,9 @@
       <c r="H50" s="3" t="n">
         <v>49</v>
       </c>
+      <c r="I50" s="3" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -2146,6 +2298,9 @@
       <c r="H51" s="3" t="n">
         <v>50</v>
       </c>
+      <c r="I51" s="3" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -2178,6 +2333,9 @@
       <c r="H52" s="3" t="n">
         <v>51</v>
       </c>
+      <c r="I52" s="3" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -2208,7 +2366,10 @@
         <v>13</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>53</v>
+        <v>52</v>
+      </c>
+      <c r="I53" s="3" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="54">
@@ -2240,7 +2401,10 @@
         <v>10</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>52</v>
+        <v>53</v>
+      </c>
+      <c r="I54" s="3" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="55">
@@ -2274,6 +2438,9 @@
       <c r="H55" s="3" t="n">
         <v>56</v>
       </c>
+      <c r="I55" s="3" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
@@ -2306,6 +2473,9 @@
       <c r="H56" s="3" t="n">
         <v>54</v>
       </c>
+      <c r="I56" s="3" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
@@ -2336,7 +2506,10 @@
         <v>17</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>55</v>
+        <v>57</v>
+      </c>
+      <c r="I57" s="3" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="58">
@@ -2368,7 +2541,10 @@
         <v>8</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>57</v>
+        <v>55</v>
+      </c>
+      <c r="I58" s="3" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="59">
@@ -2402,6 +2578,9 @@
       <c r="H59" s="3" t="n">
         <v>59</v>
       </c>
+      <c r="I59" s="3" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2432,7 +2611,10 @@
         <v>8</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>58</v>
+        <v>60</v>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>72</v>
       </c>
     </row>
     <row r="61">
@@ -2464,7 +2646,10 @@
         <v>10</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>60</v>
+        <v>58</v>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="62">
@@ -2498,6 +2683,9 @@
       <c r="H62" s="3" t="n">
         <v>63</v>
       </c>
+      <c r="I62" s="3" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2528,7 +2716,10 @@
         <v>10</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>62</v>
+        <v>61</v>
+      </c>
+      <c r="I63" s="3" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="64">
@@ -2560,7 +2751,10 @@
         <v>7</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>61</v>
+        <v>62</v>
+      </c>
+      <c r="I64" s="3" t="n">
+        <v>63</v>
       </c>
     </row>
     <row r="65">
@@ -2592,7 +2786,10 @@
         <v>6</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>67</v>
+        <v>65</v>
+      </c>
+      <c r="I65" s="3" t="n">
+        <v>71</v>
       </c>
     </row>
     <row r="66">
@@ -2624,7 +2821,10 @@
         <v>2</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>65</v>
+        <v>64</v>
+      </c>
+      <c r="I66" s="3" t="n">
+        <v>108</v>
       </c>
     </row>
     <row r="67">
@@ -2656,7 +2856,10 @@
         <v>2</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>66</v>
+        <v>67</v>
+      </c>
+      <c r="I67" s="3" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="68">
@@ -2688,7 +2891,10 @@
         <v>7</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>64</v>
+        <v>66</v>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="69">
@@ -2720,7 +2926,10 @@
         <v>5</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="I69" s="3" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="70">
@@ -2752,7 +2961,10 @@
         <v>4</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>69</v>
+        <v>68</v>
+      </c>
+      <c r="I70" s="3" t="n">
+        <v>84</v>
       </c>
     </row>
     <row r="71">
@@ -2784,7 +2996,10 @@
         <v>5</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>71</v>
+        <v>72</v>
+      </c>
+      <c r="I71" s="3" t="n">
+        <v>76</v>
       </c>
     </row>
     <row r="72">
@@ -2816,7 +3031,10 @@
         <v>4</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>73</v>
+        <v>71</v>
+      </c>
+      <c r="I72" s="3" t="n">
+        <v>78</v>
       </c>
     </row>
     <row r="73">
@@ -2848,7 +3066,10 @@
         <v>4</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>68</v>
+        <v>69</v>
+      </c>
+      <c r="I73" s="3" t="n">
+        <v>81</v>
       </c>
     </row>
     <row r="74">
@@ -2882,6 +3103,9 @@
       <c r="H74" s="3" t="n">
         <v>70</v>
       </c>
+      <c r="I74" s="3" t="n">
+        <v>79</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
@@ -2912,7 +3136,10 @@
         <v>9</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>75</v>
+        <v>77</v>
+      </c>
+      <c r="I75" s="3" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="76">
@@ -2944,7 +3171,10 @@
         <v>2</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>77</v>
+        <v>74</v>
+      </c>
+      <c r="I76" s="3" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="77">
@@ -2976,7 +3206,10 @@
         <v>11</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>74</v>
+        <v>76</v>
+      </c>
+      <c r="I77" s="3" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="78">
@@ -3008,7 +3241,10 @@
         <v>7</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="I78" s="3" t="n">
+        <v>66</v>
       </c>
     </row>
     <row r="79">
@@ -3040,7 +3276,10 @@
         <v>15</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>78</v>
+        <v>85</v>
+      </c>
+      <c r="I79" s="3" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="80">
@@ -3072,7 +3311,10 @@
         <v>2</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>82</v>
+        <v>79</v>
+      </c>
+      <c r="I80" s="3" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="81">
@@ -3104,7 +3346,10 @@
         <v>2</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>83</v>
+        <v>81</v>
+      </c>
+      <c r="I81" s="3" t="n">
+        <v>99</v>
       </c>
     </row>
     <row r="82">
@@ -3136,7 +3381,10 @@
         <v>5</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>85</v>
+        <v>86</v>
+      </c>
+      <c r="I82" s="3" t="n">
+        <v>73</v>
       </c>
     </row>
     <row r="83">
@@ -3168,7 +3416,10 @@
         <v>3</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>79</v>
+        <v>78</v>
+      </c>
+      <c r="I83" s="3" t="n">
+        <v>97</v>
       </c>
     </row>
     <row r="84">
@@ -3202,6 +3453,9 @@
       <c r="H84" s="3" t="n">
         <v>84</v>
       </c>
+      <c r="I84" s="3" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="11" t="inlineStr">
@@ -3232,7 +3486,10 @@
         <v>3</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>86</v>
+        <v>82</v>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="86">
@@ -3264,7 +3521,10 @@
         <v>2</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>80</v>
+        <v>83</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="87">
@@ -3296,7 +3556,10 @@
         <v>2</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>81</v>
+        <v>80</v>
+      </c>
+      <c r="I87" s="3" t="n">
+        <v>98</v>
       </c>
     </row>
     <row r="88">
@@ -3328,7 +3591,10 @@
         <v>6</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>90</v>
+        <v>92</v>
+      </c>
+      <c r="I88" s="3" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="89">
@@ -3360,7 +3626,10 @@
         <v>1</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>94</v>
+        <v>91</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>149</v>
       </c>
     </row>
     <row r="90">
@@ -3392,7 +3661,10 @@
         <v>1</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>95</v>
+        <v>88</v>
+      </c>
+      <c r="I90" s="3" t="n">
+        <v>136</v>
       </c>
     </row>
     <row r="91">
@@ -3424,7 +3696,10 @@
         <v>4</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>93</v>
+        <v>87</v>
+      </c>
+      <c r="I91" s="3" t="n">
+        <v>91</v>
       </c>
     </row>
     <row r="92">
@@ -3456,7 +3731,10 @@
         <v>4</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>89</v>
+        <v>94</v>
+      </c>
+      <c r="I92" s="3" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="93">
@@ -3488,7 +3766,10 @@
         <v>3</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>92</v>
+        <v>95</v>
+      </c>
+      <c r="I93" s="3" t="n">
+        <v>89</v>
       </c>
     </row>
     <row r="94">
@@ -3520,7 +3801,10 @@
         <v>5</v>
       </c>
       <c r="H94" s="3" t="n">
-        <v>91</v>
+        <v>93</v>
+      </c>
+      <c r="I94" s="3" t="n">
+        <v>77</v>
       </c>
     </row>
     <row r="95">
@@ -3552,7 +3836,10 @@
         <v>2</v>
       </c>
       <c r="H95" s="3" t="n">
-        <v>88</v>
+        <v>89</v>
+      </c>
+      <c r="I95" s="3" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="96">
@@ -3584,7 +3871,10 @@
         <v>7</v>
       </c>
       <c r="H96" s="3" t="n">
-        <v>87</v>
+        <v>90</v>
+      </c>
+      <c r="I96" s="3" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="97">
@@ -3616,7 +3906,10 @@
         <v>6</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>120</v>
+        <v>111</v>
+      </c>
+      <c r="I97" s="3" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="98">
@@ -3648,7 +3941,10 @@
         <v>2</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>106</v>
+        <v>118</v>
+      </c>
+      <c r="I98" s="3" t="n">
+        <v>111</v>
       </c>
     </row>
     <row r="99">
@@ -3682,6 +3978,9 @@
       <c r="H99" s="3" t="n">
         <v>116</v>
       </c>
+      <c r="I99" s="3" t="n">
+        <v>137</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3712,7 +4011,10 @@
         <v>4</v>
       </c>
       <c r="H100" s="3" t="n">
-        <v>102</v>
+        <v>96</v>
+      </c>
+      <c r="I100" s="3" t="n">
+        <v>86</v>
       </c>
     </row>
     <row r="101">
@@ -3746,6 +4048,9 @@
       <c r="H101" s="3" t="n">
         <v>115</v>
       </c>
+      <c r="I101" s="3" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
@@ -3776,7 +4081,10 @@
         <v>1</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>107</v>
+        <v>99</v>
+      </c>
+      <c r="I102" s="3" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="103">
@@ -3808,7 +4116,10 @@
         <v>4</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>118</v>
+        <v>112</v>
+      </c>
+      <c r="I103" s="3" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="104">
@@ -3840,7 +4151,10 @@
         <v>1</v>
       </c>
       <c r="H104" s="3" t="n">
-        <v>110</v>
+        <v>104</v>
+      </c>
+      <c r="I104" s="3" t="n">
+        <v>121</v>
       </c>
     </row>
     <row r="105">
@@ -3872,7 +4186,10 @@
         <v>1</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>108</v>
+        <v>98</v>
+      </c>
+      <c r="I105" s="3" t="n">
+        <v>131</v>
       </c>
     </row>
     <row r="106">
@@ -3904,7 +4221,10 @@
         <v>3</v>
       </c>
       <c r="H106" s="3" t="n">
-        <v>98</v>
+        <v>114</v>
+      </c>
+      <c r="I106" s="3" t="n">
+        <v>87</v>
       </c>
     </row>
     <row r="107">
@@ -3936,7 +4256,10 @@
         <v>3</v>
       </c>
       <c r="H107" s="3" t="n">
-        <v>99</v>
+        <v>113</v>
+      </c>
+      <c r="I107" s="3" t="n">
+        <v>93</v>
       </c>
     </row>
     <row r="108">
@@ -3968,7 +4291,10 @@
         <v>3</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>101</v>
+        <v>97</v>
+      </c>
+      <c r="I108" s="3" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="109">
@@ -4000,7 +4326,10 @@
         <v>2</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>111</v>
+        <v>106</v>
+      </c>
+      <c r="I109" s="3" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="110">
@@ -4032,7 +4361,10 @@
         <v>1</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>114</v>
+        <v>119</v>
+      </c>
+      <c r="I110" s="3" t="n">
+        <v>152</v>
       </c>
     </row>
     <row r="111">
@@ -4064,7 +4396,10 @@
         <v>1</v>
       </c>
       <c r="H111" s="3" t="n">
-        <v>96</v>
+        <v>103</v>
+      </c>
+      <c r="I111" s="3" t="n">
+        <v>122</v>
       </c>
     </row>
     <row r="112">
@@ -4096,7 +4431,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="3" t="n">
-        <v>119</v>
+        <v>108</v>
+      </c>
+      <c r="I112" s="3" t="n">
+        <v>217</v>
       </c>
     </row>
     <row r="113">
@@ -4128,7 +4466,10 @@
         <v>1</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>117</v>
+        <v>120</v>
+      </c>
+      <c r="I113" s="3" t="n">
+        <v>148</v>
       </c>
     </row>
     <row r="114">
@@ -4160,7 +4501,10 @@
         <v>2</v>
       </c>
       <c r="H114" s="3" t="n">
-        <v>105</v>
+        <v>110</v>
+      </c>
+      <c r="I114" s="3" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="115">
@@ -4192,7 +4536,10 @@
         <v>4</v>
       </c>
       <c r="H115" s="3" t="n">
-        <v>103</v>
+        <v>105</v>
+      </c>
+      <c r="I115" s="3" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="116">
@@ -4224,7 +4571,10 @@
         <v>3</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>100</v>
+        <v>117</v>
+      </c>
+      <c r="I116" s="3" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="117">
@@ -4256,7 +4606,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>112</v>
+        <v>109</v>
+      </c>
+      <c r="I117" s="3" t="n">
+        <v>260</v>
       </c>
     </row>
     <row r="118">
@@ -4288,7 +4641,10 @@
         <v>1</v>
       </c>
       <c r="H118" s="3" t="n">
-        <v>97</v>
+        <v>100</v>
+      </c>
+      <c r="I118" s="3" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="119">
@@ -4320,7 +4676,10 @@
         <v>2</v>
       </c>
       <c r="H119" s="3" t="n">
-        <v>104</v>
+        <v>107</v>
+      </c>
+      <c r="I119" s="3" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="120">
@@ -4352,7 +4711,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="3" t="n">
-        <v>113</v>
+        <v>101</v>
+      </c>
+      <c r="I120" s="3" t="n">
+        <v>183</v>
       </c>
     </row>
     <row r="121">
@@ -4384,7 +4746,10 @@
         <v>1</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>109</v>
+        <v>102</v>
+      </c>
+      <c r="I121" s="3" t="n">
+        <v>88</v>
       </c>
     </row>
     <row r="122">
@@ -4416,7 +4781,10 @@
         <v>3</v>
       </c>
       <c r="H122" s="3" t="n">
-        <v>123</v>
+        <v>158</v>
+      </c>
+      <c r="I122" s="3" t="n">
+        <v>94</v>
       </c>
     </row>
     <row r="123">
@@ -4448,7 +4816,10 @@
         <v>1</v>
       </c>
       <c r="H123" s="3" t="n">
-        <v>138</v>
+        <v>159</v>
+      </c>
+      <c r="I123" s="3" t="n">
+        <v>147</v>
       </c>
     </row>
     <row r="124">
@@ -4480,7 +4851,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="3" t="n">
-        <v>128</v>
+        <v>141</v>
+      </c>
+      <c r="I124" s="3" t="n">
+        <v>190</v>
       </c>
     </row>
     <row r="125">
@@ -4512,7 +4886,10 @@
         <v>3</v>
       </c>
       <c r="H125" s="3" t="n">
-        <v>121</v>
+        <v>160</v>
+      </c>
+      <c r="I125" s="3" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="126">
@@ -4544,7 +4921,10 @@
         <v>2</v>
       </c>
       <c r="H126" s="3" t="n">
-        <v>132</v>
+        <v>152</v>
+      </c>
+      <c r="I126" s="3" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="127">
@@ -4576,7 +4956,10 @@
         <v>1</v>
       </c>
       <c r="H127" s="3" t="n">
-        <v>141</v>
+        <v>143</v>
+      </c>
+      <c r="I127" s="3" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="128">
@@ -4608,7 +4991,10 @@
         <v>2</v>
       </c>
       <c r="H128" s="3" t="n">
-        <v>126</v>
+        <v>157</v>
+      </c>
+      <c r="I128" s="3" t="n">
+        <v>101</v>
       </c>
     </row>
     <row r="129">
@@ -4640,7 +5026,10 @@
         <v>1</v>
       </c>
       <c r="H129" s="3" t="n">
-        <v>143</v>
+        <v>145</v>
+      </c>
+      <c r="I129" s="3" t="n">
+        <v>135</v>
       </c>
     </row>
     <row r="130">
@@ -4672,7 +5061,10 @@
         <v>1</v>
       </c>
       <c r="H130" s="3" t="n">
-        <v>135</v>
+        <v>153</v>
+      </c>
+      <c r="I130" s="3" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="131">
@@ -4704,7 +5096,10 @@
         <v>2</v>
       </c>
       <c r="H131" s="3" t="n">
-        <v>125</v>
+        <v>150</v>
+      </c>
+      <c r="I131" s="3" t="n">
+        <v>110</v>
       </c>
     </row>
     <row r="132">
@@ -4736,7 +5131,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="3" t="n">
-        <v>146</v>
+        <v>133</v>
+      </c>
+      <c r="I132" s="3" t="n">
+        <v>198</v>
       </c>
     </row>
     <row r="133">
@@ -4768,7 +5166,10 @@
         <v>1</v>
       </c>
       <c r="H133" s="3" t="n">
-        <v>159</v>
+        <v>144</v>
+      </c>
+      <c r="I133" s="3" t="n">
+        <v>134</v>
       </c>
     </row>
     <row r="134">
@@ -4800,7 +5201,10 @@
         <v>2</v>
       </c>
       <c r="H134" s="3" t="n">
-        <v>122</v>
+        <v>149</v>
+      </c>
+      <c r="I134" s="3" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="135">
@@ -4832,7 +5236,10 @@
         <v>0</v>
       </c>
       <c r="H135" s="3" t="n">
-        <v>145</v>
+        <v>128</v>
+      </c>
+      <c r="I135" s="3" t="n">
+        <v>166</v>
       </c>
     </row>
     <row r="136">
@@ -4864,7 +5271,10 @@
         <v>2</v>
       </c>
       <c r="H136" s="3" t="n">
-        <v>136</v>
+        <v>148</v>
+      </c>
+      <c r="I136" s="3" t="n">
+        <v>114</v>
       </c>
     </row>
     <row r="137">
@@ -4896,7 +5306,10 @@
         <v>0</v>
       </c>
       <c r="H137" s="3" t="n">
-        <v>148</v>
+        <v>121</v>
+      </c>
+      <c r="I137" s="3" t="n">
+        <v>178</v>
       </c>
     </row>
     <row r="138">
@@ -4928,7 +5341,10 @@
         <v>2</v>
       </c>
       <c r="H138" s="3" t="n">
-        <v>124</v>
+        <v>156</v>
+      </c>
+      <c r="I138" s="3" t="n">
+        <v>104</v>
       </c>
     </row>
     <row r="139">
@@ -4960,7 +5376,10 @@
         <v>0</v>
       </c>
       <c r="H139" s="3" t="n">
-        <v>149</v>
+        <v>130</v>
+      </c>
+      <c r="I139" s="3" t="n">
+        <v>186</v>
       </c>
     </row>
     <row r="140">
@@ -4992,7 +5411,10 @@
         <v>0</v>
       </c>
       <c r="H140" s="3" t="n">
-        <v>144</v>
+        <v>122</v>
+      </c>
+      <c r="I140" s="3" t="n">
+        <v>171</v>
       </c>
     </row>
     <row r="141">
@@ -5024,7 +5446,10 @@
         <v>2</v>
       </c>
       <c r="H141" s="3" t="n">
-        <v>127</v>
+        <v>154</v>
+      </c>
+      <c r="I141" s="3" t="n">
+        <v>112</v>
       </c>
     </row>
     <row r="142">
@@ -5056,7 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>137</v>
+        <v>123</v>
+      </c>
+      <c r="I142" s="3" t="n">
+        <v>170</v>
       </c>
     </row>
     <row r="143">
@@ -5088,7 +5516,10 @@
         <v>0</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>139</v>
+        <v>126</v>
+      </c>
+      <c r="I143" s="3" t="n">
+        <v>156</v>
       </c>
     </row>
     <row r="144">
@@ -5120,6 +5551,9 @@
         <v>1</v>
       </c>
       <c r="H144" s="3" t="n">
+        <v>139</v>
+      </c>
+      <c r="I144" s="3" t="n">
         <v>158</v>
       </c>
     </row>
@@ -5152,7 +5586,10 @@
         <v>0</v>
       </c>
       <c r="H145" s="3" t="n">
-        <v>151</v>
+        <v>135</v>
+      </c>
+      <c r="I145" s="3" t="n">
+        <v>216</v>
       </c>
     </row>
     <row r="146">
@@ -5184,7 +5621,10 @@
         <v>0</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>156</v>
+        <v>137</v>
+      </c>
+      <c r="I146" s="3" t="n">
+        <v>181</v>
       </c>
     </row>
     <row r="147">
@@ -5216,7 +5656,10 @@
         <v>1</v>
       </c>
       <c r="H147" s="3" t="n">
-        <v>140</v>
+        <v>125</v>
+      </c>
+      <c r="I147" s="3" t="n">
+        <v>151</v>
       </c>
     </row>
     <row r="148">
@@ -5248,7 +5691,10 @@
         <v>0</v>
       </c>
       <c r="H148" s="3" t="n">
-        <v>147</v>
+        <v>132</v>
+      </c>
+      <c r="I148" s="3" t="n">
+        <v>197</v>
       </c>
     </row>
     <row r="149">
@@ -5280,7 +5726,10 @@
         <v>2</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>134</v>
+        <v>151</v>
+      </c>
+      <c r="I149" s="3" t="n">
+        <v>126</v>
       </c>
     </row>
     <row r="150">
@@ -5312,7 +5761,10 @@
         <v>2</v>
       </c>
       <c r="H150" s="3" t="n">
-        <v>133</v>
+        <v>146</v>
+      </c>
+      <c r="I150" s="3" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="151">
@@ -5344,7 +5796,10 @@
         <v>1</v>
       </c>
       <c r="H151" s="3" t="n">
-        <v>131</v>
+        <v>147</v>
+      </c>
+      <c r="I151" s="3" t="n">
+        <v>133</v>
       </c>
     </row>
     <row r="152">
@@ -5376,7 +5831,10 @@
         <v>0</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>160</v>
+        <v>138</v>
+      </c>
+      <c r="I152" s="3" t="n">
+        <v>223</v>
       </c>
     </row>
     <row r="153">
@@ -5408,7 +5866,10 @@
         <v>0</v>
       </c>
       <c r="H153" s="3" t="n">
-        <v>129</v>
+        <v>142</v>
+      </c>
+      <c r="I153" s="3" t="n">
+        <v>268</v>
       </c>
     </row>
     <row r="154">
@@ -5440,7 +5901,10 @@
         <v>0</v>
       </c>
       <c r="H154" s="3" t="n">
-        <v>152</v>
+        <v>129</v>
+      </c>
+      <c r="I154" s="3" t="n">
+        <v>213</v>
       </c>
     </row>
     <row r="155">
@@ -5472,7 +5936,10 @@
         <v>0</v>
       </c>
       <c r="H155" s="3" t="n">
-        <v>150</v>
+        <v>134</v>
+      </c>
+      <c r="I155" s="3" t="n">
+        <v>192</v>
       </c>
     </row>
     <row r="156">
@@ -5506,6 +5973,9 @@
       <c r="H156" s="3" t="n">
         <v>155</v>
       </c>
+      <c r="I156" s="3" t="n">
+        <v>155</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -5536,7 +6006,10 @@
         <v>0</v>
       </c>
       <c r="H157" s="3" t="n">
-        <v>157</v>
+        <v>136</v>
+      </c>
+      <c r="I157" s="3" t="n">
+        <v>209</v>
       </c>
     </row>
     <row r="158">
@@ -5568,7 +6041,10 @@
         <v>0</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>142</v>
+        <v>124</v>
+      </c>
+      <c r="I158" s="3" t="n">
+        <v>169</v>
       </c>
     </row>
     <row r="159">
@@ -5600,7 +6076,10 @@
         <v>0</v>
       </c>
       <c r="H159" s="3" t="n">
-        <v>153</v>
+        <v>131</v>
+      </c>
+      <c r="I159" s="3" t="n">
+        <v>194</v>
       </c>
     </row>
     <row r="160">
@@ -5632,7 +6111,10 @@
         <v>0</v>
       </c>
       <c r="H160" s="3" t="n">
-        <v>130</v>
+        <v>140</v>
+      </c>
+      <c r="I160" s="3" t="n">
+        <v>235</v>
       </c>
     </row>
     <row r="161">
@@ -5664,7 +6146,10 @@
         <v>0</v>
       </c>
       <c r="H161" s="3" t="n">
-        <v>154</v>
+        <v>127</v>
+      </c>
+      <c r="I161" s="3" t="n">
+        <v>172</v>
       </c>
     </row>
     <row r="162">
@@ -5696,7 +6181,10 @@
         <v>1</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>164</v>
+        <v>167</v>
+      </c>
+      <c r="I162" s="3" t="n">
+        <v>157</v>
       </c>
     </row>
     <row r="163">
@@ -5728,7 +6216,10 @@
         <v>0</v>
       </c>
       <c r="H163" s="3" t="n">
-        <v>177</v>
+        <v>231</v>
+      </c>
+      <c r="I163" s="3" t="n">
+        <v>199</v>
       </c>
     </row>
     <row r="164">
@@ -5760,7 +6251,10 @@
         <v>0</v>
       </c>
       <c r="H164" s="3" t="n">
-        <v>192</v>
+        <v>243</v>
+      </c>
+      <c r="I164" s="3" t="n">
+        <v>215</v>
       </c>
     </row>
     <row r="165">
@@ -5792,7 +6286,10 @@
         <v>0</v>
       </c>
       <c r="H165" s="3" t="n">
-        <v>179</v>
+        <v>233</v>
+      </c>
+      <c r="I165" s="3" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="166">
@@ -5824,7 +6321,10 @@
         <v>0</v>
       </c>
       <c r="H166" s="3" t="n">
-        <v>240</v>
+        <v>196</v>
+      </c>
+      <c r="I166" s="3" t="n">
+        <v>262</v>
       </c>
     </row>
     <row r="167">
@@ -5856,7 +6356,10 @@
         <v>0</v>
       </c>
       <c r="H167" s="3" t="n">
-        <v>175</v>
+        <v>218</v>
+      </c>
+      <c r="I167" s="3" t="n">
+        <v>195</v>
       </c>
     </row>
     <row r="168">
@@ -5888,7 +6391,10 @@
         <v>0</v>
       </c>
       <c r="H168" s="3" t="n">
-        <v>201</v>
+        <v>239</v>
+      </c>
+      <c r="I168" s="3" t="n">
+        <v>225</v>
       </c>
     </row>
     <row r="169">
@@ -5920,7 +6426,10 @@
         <v>1</v>
       </c>
       <c r="H169" s="3" t="n">
-        <v>161</v>
+        <v>211</v>
+      </c>
+      <c r="I169" s="3" t="n">
+        <v>123</v>
       </c>
     </row>
     <row r="170">
@@ -5952,7 +6461,10 @@
         <v>2</v>
       </c>
       <c r="H170" s="3" t="n">
-        <v>162</v>
+        <v>235</v>
+      </c>
+      <c r="I170" s="3" t="n">
+        <v>107</v>
       </c>
     </row>
     <row r="171">
@@ -5984,7 +6496,10 @@
         <v>1</v>
       </c>
       <c r="H171" s="3" t="n">
-        <v>189</v>
+        <v>220</v>
+      </c>
+      <c r="I171" s="3" t="n">
+        <v>140</v>
       </c>
     </row>
     <row r="172">
@@ -6016,7 +6531,10 @@
         <v>1</v>
       </c>
       <c r="H172" s="3" t="n">
-        <v>167</v>
+        <v>230</v>
+      </c>
+      <c r="I172" s="3" t="n">
+        <v>153</v>
       </c>
     </row>
     <row r="173">
@@ -6048,7 +6566,10 @@
         <v>0</v>
       </c>
       <c r="H173" s="3" t="n">
-        <v>169</v>
+        <v>226</v>
+      </c>
+      <c r="I173" s="3" t="n">
+        <v>164</v>
       </c>
     </row>
     <row r="174">
@@ -6080,7 +6601,10 @@
         <v>1</v>
       </c>
       <c r="H174" s="3" t="n">
-        <v>190</v>
+        <v>221</v>
+      </c>
+      <c r="I174" s="3" t="n">
+        <v>141</v>
       </c>
     </row>
     <row r="175">
@@ -6112,7 +6636,10 @@
         <v>0</v>
       </c>
       <c r="H175" s="3" t="n">
-        <v>171</v>
+        <v>227</v>
+      </c>
+      <c r="I175" s="3" t="n">
+        <v>163</v>
       </c>
     </row>
     <row r="176">
@@ -6144,7 +6671,10 @@
         <v>0</v>
       </c>
       <c r="H176" s="3" t="n">
-        <v>182</v>
+        <v>254</v>
+      </c>
+      <c r="I176" s="3" t="n">
+        <v>202</v>
       </c>
     </row>
     <row r="177">
@@ -6176,7 +6706,10 @@
         <v>1</v>
       </c>
       <c r="H177" s="3" t="n">
-        <v>188</v>
+        <v>219</v>
+      </c>
+      <c r="I177" s="3" t="n">
+        <v>139</v>
       </c>
     </row>
     <row r="178">
@@ -6208,7 +6741,10 @@
         <v>1</v>
       </c>
       <c r="H178" s="3" t="n">
-        <v>185</v>
+        <v>222</v>
+      </c>
+      <c r="I178" s="3" t="n">
+        <v>145</v>
       </c>
     </row>
     <row r="179">
@@ -6240,7 +6776,10 @@
         <v>0</v>
       </c>
       <c r="H179" s="3" t="n">
-        <v>166</v>
+        <v>228</v>
+      </c>
+      <c r="I179" s="3" t="n">
+        <v>162</v>
       </c>
     </row>
     <row r="180">
@@ -6272,7 +6811,10 @@
         <v>1</v>
       </c>
       <c r="H180" s="3" t="n">
-        <v>165</v>
+        <v>229</v>
+      </c>
+      <c r="I180" s="3" t="n">
+        <v>161</v>
       </c>
     </row>
     <row r="181">
@@ -6304,7 +6846,10 @@
         <v>0</v>
       </c>
       <c r="H181" s="3" t="n">
-        <v>203</v>
+        <v>207</v>
+      </c>
+      <c r="I181" s="3" t="n">
+        <v>228</v>
       </c>
     </row>
     <row r="182">
@@ -6336,7 +6881,10 @@
         <v>0</v>
       </c>
       <c r="H182" s="3" t="n">
-        <v>222</v>
+        <v>164</v>
+      </c>
+      <c r="I182" s="3" t="n">
+        <v>253</v>
       </c>
     </row>
     <row r="183">
@@ -6368,7 +6916,10 @@
         <v>0</v>
       </c>
       <c r="H183" s="3" t="n">
-        <v>186</v>
+        <v>213</v>
+      </c>
+      <c r="I183" s="3" t="n">
+        <v>185</v>
       </c>
     </row>
     <row r="184">
@@ -6400,7 +6951,10 @@
         <v>0</v>
       </c>
       <c r="H184" s="3" t="n">
-        <v>216</v>
+        <v>173</v>
+      </c>
+      <c r="I184" s="3" t="n">
+        <v>243</v>
       </c>
     </row>
     <row r="185">
@@ -6432,7 +6986,10 @@
         <v>0</v>
       </c>
       <c r="H185" s="3" t="n">
-        <v>215</v>
+        <v>177</v>
+      </c>
+      <c r="I185" s="3" t="n">
+        <v>239</v>
       </c>
     </row>
     <row r="186">
@@ -6464,7 +7021,10 @@
         <v>0</v>
       </c>
       <c r="H186" s="3" t="n">
-        <v>226</v>
+        <v>165</v>
+      </c>
+      <c r="I186" s="3" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="187">
@@ -6496,7 +7056,10 @@
         <v>2</v>
       </c>
       <c r="H187" s="3" t="n">
-        <v>163</v>
+        <v>244</v>
+      </c>
+      <c r="I187" s="3" t="n">
+        <v>115</v>
       </c>
     </row>
     <row r="188">
@@ -6528,7 +7091,10 @@
         <v>0</v>
       </c>
       <c r="H188" s="3" t="n">
-        <v>183</v>
+        <v>253</v>
+      </c>
+      <c r="I188" s="3" t="n">
+        <v>206</v>
       </c>
     </row>
     <row r="189">
@@ -6560,7 +7126,10 @@
         <v>0</v>
       </c>
       <c r="H189" s="3" t="n">
-        <v>168</v>
+        <v>225</v>
+      </c>
+      <c r="I189" s="3" t="n">
+        <v>165</v>
       </c>
     </row>
     <row r="190">
@@ -6592,7 +7161,10 @@
         <v>0</v>
       </c>
       <c r="H190" s="3" t="n">
-        <v>228</v>
+        <v>170</v>
+      </c>
+      <c r="I190" s="3" t="n">
+        <v>274</v>
       </c>
     </row>
     <row r="191">
@@ -6624,7 +7196,10 @@
         <v>1</v>
       </c>
       <c r="H191" s="3" t="n">
-        <v>184</v>
+        <v>215</v>
+      </c>
+      <c r="I191" s="3" t="n">
+        <v>92</v>
       </c>
     </row>
     <row r="192">
@@ -6656,7 +7231,10 @@
         <v>0</v>
       </c>
       <c r="H192" s="3" t="n">
-        <v>176</v>
+        <v>232</v>
+      </c>
+      <c r="I192" s="3" t="n">
+        <v>180</v>
       </c>
     </row>
     <row r="193">
@@ -6688,7 +7266,10 @@
         <v>0</v>
       </c>
       <c r="H193" s="3" t="n">
-        <v>235</v>
+        <v>201</v>
+      </c>
+      <c r="I193" s="3" t="n">
+        <v>275</v>
       </c>
     </row>
     <row r="194">
@@ -6720,7 +7301,10 @@
         <v>0</v>
       </c>
       <c r="H194" s="3" t="n">
-        <v>232</v>
+        <v>204</v>
+      </c>
+      <c r="I194" s="3" t="n">
+        <v>272</v>
       </c>
     </row>
     <row r="195">
@@ -6752,7 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H195" s="3" t="n">
-        <v>206</v>
+        <v>241</v>
+      </c>
+      <c r="I195" s="3" t="n">
+        <v>219</v>
       </c>
     </row>
     <row r="196">
@@ -6784,7 +7371,10 @@
         <v>0</v>
       </c>
       <c r="H196" s="3" t="n">
-        <v>219</v>
+        <v>171</v>
+      </c>
+      <c r="I196" s="3" t="n">
+        <v>244</v>
       </c>
     </row>
     <row r="197">
@@ -6816,7 +7406,10 @@
         <v>0</v>
       </c>
       <c r="H197" s="3" t="n">
-        <v>193</v>
+        <v>234</v>
+      </c>
+      <c r="I197" s="3" t="n">
+        <v>214</v>
       </c>
     </row>
     <row r="198">
@@ -6848,7 +7441,10 @@
         <v>0</v>
       </c>
       <c r="H198" s="3" t="n">
-        <v>227</v>
+        <v>178</v>
+      </c>
+      <c r="I198" s="3" t="n">
+        <v>269</v>
       </c>
     </row>
     <row r="199">
@@ -6880,7 +7476,10 @@
         <v>0</v>
       </c>
       <c r="H199" s="3" t="n">
-        <v>205</v>
+        <v>236</v>
+      </c>
+      <c r="I199" s="3" t="n">
+        <v>210</v>
       </c>
     </row>
     <row r="200">
@@ -6912,7 +7511,10 @@
         <v>0</v>
       </c>
       <c r="H200" s="3" t="n">
-        <v>196</v>
+        <v>248</v>
+      </c>
+      <c r="I200" s="3" t="n">
+        <v>211</v>
       </c>
     </row>
     <row r="201">
@@ -6944,7 +7546,10 @@
         <v>0</v>
       </c>
       <c r="H201" s="3" t="n">
-        <v>204</v>
+        <v>237</v>
+      </c>
+      <c r="I201" s="3" t="n">
+        <v>224</v>
       </c>
     </row>
     <row r="202">
@@ -6978,6 +7583,9 @@
       <c r="H202" s="3" t="n">
         <v>209</v>
       </c>
+      <c r="I202" s="3" t="n">
+        <v>236</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="8" t="inlineStr">
@@ -7008,7 +7616,10 @@
         <v>0</v>
       </c>
       <c r="H203" s="3" t="n">
-        <v>174</v>
+        <v>217</v>
+      </c>
+      <c r="I203" s="3" t="n">
+        <v>173</v>
       </c>
     </row>
     <row r="204">
@@ -7040,7 +7651,10 @@
         <v>0</v>
       </c>
       <c r="H204" s="3" t="n">
-        <v>173</v>
+        <v>214</v>
+      </c>
+      <c r="I204" s="3" t="n">
+        <v>184</v>
       </c>
     </row>
     <row r="205">
@@ -7072,7 +7686,10 @@
         <v>0</v>
       </c>
       <c r="H205" s="3" t="n">
-        <v>170</v>
+        <v>223</v>
+      </c>
+      <c r="I205" s="3" t="n">
+        <v>167</v>
       </c>
     </row>
     <row r="206">
@@ -7104,7 +7721,10 @@
         <v>0</v>
       </c>
       <c r="H206" s="3" t="n">
-        <v>187</v>
+        <v>216</v>
+      </c>
+      <c r="I206" s="3" t="n">
+        <v>177</v>
       </c>
     </row>
     <row r="207">
@@ -7136,7 +7756,10 @@
         <v>0</v>
       </c>
       <c r="H207" s="3" t="n">
-        <v>197</v>
+        <v>251</v>
+      </c>
+      <c r="I207" s="3" t="n">
+        <v>208</v>
       </c>
     </row>
     <row r="208">
@@ -7168,7 +7791,10 @@
         <v>0</v>
       </c>
       <c r="H208" s="3" t="n">
-        <v>238</v>
+        <v>198</v>
+      </c>
+      <c r="I208" s="3" t="n">
+        <v>279</v>
       </c>
     </row>
     <row r="209">
@@ -7200,7 +7826,10 @@
         <v>0</v>
       </c>
       <c r="H209" s="3" t="n">
-        <v>244</v>
+        <v>192</v>
+      </c>
+      <c r="I209" s="3" t="n">
+        <v>287</v>
       </c>
     </row>
     <row r="210">
@@ -7232,7 +7861,10 @@
         <v>0</v>
       </c>
       <c r="H210" s="3" t="n">
-        <v>231</v>
+        <v>179</v>
+      </c>
+      <c r="I210" s="3" t="n">
+        <v>252</v>
       </c>
     </row>
     <row r="211">
@@ -7264,7 +7896,10 @@
         <v>0</v>
       </c>
       <c r="H211" s="3" t="n">
-        <v>194</v>
+        <v>247</v>
+      </c>
+      <c r="I211" s="3" t="n">
+        <v>196</v>
       </c>
     </row>
     <row r="212">
@@ -7296,7 +7931,10 @@
         <v>0</v>
       </c>
       <c r="H212" s="3" t="n">
-        <v>239</v>
+        <v>197</v>
+      </c>
+      <c r="I212" s="3" t="n">
+        <v>280</v>
       </c>
     </row>
     <row r="213">
@@ -7328,7 +7966,10 @@
         <v>0</v>
       </c>
       <c r="H213" s="3" t="n">
-        <v>241</v>
+        <v>195</v>
+      </c>
+      <c r="I213" s="3" t="n">
+        <v>281</v>
       </c>
     </row>
     <row r="214">
@@ -7360,7 +8001,10 @@
         <v>0</v>
       </c>
       <c r="H214" s="3" t="n">
-        <v>236</v>
+        <v>200</v>
+      </c>
+      <c r="I214" s="3" t="n">
+        <v>278</v>
       </c>
     </row>
     <row r="215">
@@ -7394,6 +8038,9 @@
       <c r="H215" s="3" t="n">
         <v>208</v>
       </c>
+      <c r="I215" s="3" t="n">
+        <v>237</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="6" t="inlineStr">
@@ -7424,7 +8071,10 @@
         <v>0</v>
       </c>
       <c r="H216" s="3" t="n">
-        <v>211</v>
+        <v>205</v>
+      </c>
+      <c r="I216" s="3" t="n">
+        <v>238</v>
       </c>
     </row>
     <row r="217">
@@ -7456,7 +8106,10 @@
         <v>0</v>
       </c>
       <c r="H217" s="3" t="n">
-        <v>210</v>
+        <v>206</v>
+      </c>
+      <c r="I217" s="3" t="n">
+        <v>248</v>
       </c>
     </row>
     <row r="218">
@@ -7488,7 +8141,10 @@
         <v>0</v>
       </c>
       <c r="H218" s="3" t="n">
-        <v>253</v>
+        <v>183</v>
+      </c>
+      <c r="I218" s="3" t="n">
+        <v>246</v>
       </c>
     </row>
     <row r="219">
@@ -7520,7 +8176,10 @@
         <v>0</v>
       </c>
       <c r="H219" s="3" t="n">
-        <v>242</v>
+        <v>193</v>
+      </c>
+      <c r="I219" s="3" t="n">
+        <v>283</v>
       </c>
     </row>
     <row r="220">
@@ -7552,7 +8211,10 @@
         <v>0</v>
       </c>
       <c r="H220" s="3" t="n">
-        <v>243</v>
+        <v>181</v>
+      </c>
+      <c r="I220" s="3" t="n">
+        <v>288</v>
       </c>
     </row>
     <row r="221">
@@ -7584,7 +8246,10 @@
         <v>0</v>
       </c>
       <c r="H221" s="3" t="n">
-        <v>181</v>
+        <v>245</v>
+      </c>
+      <c r="I221" s="3" t="n">
+        <v>201</v>
       </c>
     </row>
     <row r="222">
@@ -7616,7 +8281,10 @@
         <v>0</v>
       </c>
       <c r="H222" s="3" t="n">
-        <v>178</v>
+        <v>212</v>
+      </c>
+      <c r="I222" s="3" t="n">
+        <v>187</v>
       </c>
     </row>
     <row r="223">
@@ -7648,7 +8316,10 @@
         <v>0</v>
       </c>
       <c r="H223" s="3" t="n">
-        <v>250</v>
+        <v>186</v>
+      </c>
+      <c r="I223" s="3" t="n">
+        <v>285</v>
       </c>
     </row>
     <row r="224">
@@ -7680,7 +8351,10 @@
         <v>0</v>
       </c>
       <c r="H224" s="3" t="n">
-        <v>251</v>
+        <v>185</v>
+      </c>
+      <c r="I224" s="3" t="n">
+        <v>286</v>
       </c>
     </row>
     <row r="225">
@@ -7712,7 +8386,10 @@
         <v>0</v>
       </c>
       <c r="H225" s="3" t="n">
-        <v>198</v>
+        <v>250</v>
+      </c>
+      <c r="I225" s="3" t="n">
+        <v>168</v>
       </c>
     </row>
     <row r="226">
@@ -7744,7 +8421,10 @@
         <v>0</v>
       </c>
       <c r="H226" s="3" t="n">
-        <v>223</v>
+        <v>162</v>
+      </c>
+      <c r="I226" s="3" t="n">
+        <v>193</v>
       </c>
     </row>
     <row r="227">
@@ -7776,7 +8456,10 @@
         <v>0</v>
       </c>
       <c r="H227" s="3" t="n">
-        <v>247</v>
+        <v>189</v>
+      </c>
+      <c r="I227" s="3" t="n">
+        <v>276</v>
       </c>
     </row>
     <row r="228">
@@ -7808,7 +8491,10 @@
         <v>0</v>
       </c>
       <c r="H228" s="3" t="n">
-        <v>229</v>
+        <v>180</v>
+      </c>
+      <c r="I228" s="3" t="n">
+        <v>266</v>
       </c>
     </row>
     <row r="229">
@@ -7840,7 +8526,10 @@
         <v>0</v>
       </c>
       <c r="H229" s="3" t="n">
-        <v>246</v>
+        <v>190</v>
+      </c>
+      <c r="I229" s="3" t="n">
+        <v>289</v>
       </c>
     </row>
     <row r="230">
@@ -7872,7 +8561,10 @@
         <v>0</v>
       </c>
       <c r="H230" s="3" t="n">
-        <v>230</v>
+        <v>194</v>
+      </c>
+      <c r="I230" s="3" t="n">
+        <v>265</v>
       </c>
     </row>
     <row r="231">
@@ -7904,7 +8596,10 @@
         <v>0</v>
       </c>
       <c r="H231" s="3" t="n">
-        <v>248</v>
+        <v>188</v>
+      </c>
+      <c r="I231" s="3" t="n">
+        <v>290</v>
       </c>
     </row>
     <row r="232">
@@ -7936,7 +8631,10 @@
         <v>0</v>
       </c>
       <c r="H232" s="3" t="n">
-        <v>199</v>
+        <v>249</v>
+      </c>
+      <c r="I232" s="3" t="n">
+        <v>191</v>
       </c>
     </row>
     <row r="233">
@@ -7968,7 +8666,10 @@
         <v>0</v>
       </c>
       <c r="H233" s="3" t="n">
-        <v>233</v>
+        <v>203</v>
+      </c>
+      <c r="I233" s="3" t="n">
+        <v>273</v>
       </c>
     </row>
     <row r="234">
@@ -8000,7 +8701,10 @@
         <v>0</v>
       </c>
       <c r="H234" s="3" t="n">
-        <v>217</v>
+        <v>172</v>
+      </c>
+      <c r="I234" s="3" t="n">
+        <v>179</v>
       </c>
     </row>
     <row r="235">
@@ -8032,7 +8736,10 @@
         <v>1</v>
       </c>
       <c r="H235" s="3" t="n">
-        <v>191</v>
+        <v>224</v>
+      </c>
+      <c r="I235" s="3" t="n">
+        <v>146</v>
       </c>
     </row>
     <row r="236">
@@ -8064,7 +8771,10 @@
         <v>0</v>
       </c>
       <c r="H236" s="3" t="n">
-        <v>172</v>
+        <v>210</v>
+      </c>
+      <c r="I236" s="3" t="n">
+        <v>220</v>
       </c>
     </row>
     <row r="237">
@@ -8096,7 +8806,10 @@
         <v>0</v>
       </c>
       <c r="H237" s="3" t="n">
-        <v>207</v>
+        <v>242</v>
+      </c>
+      <c r="I237" s="3" t="n">
+        <v>218</v>
       </c>
     </row>
     <row r="238">
@@ -8128,7 +8841,10 @@
         <v>0</v>
       </c>
       <c r="H238" s="3" t="n">
-        <v>200</v>
+        <v>238</v>
+      </c>
+      <c r="I238" s="3" t="n">
+        <v>227</v>
       </c>
     </row>
     <row r="239">
@@ -8160,7 +8876,10 @@
         <v>0</v>
       </c>
       <c r="H239" s="3" t="n">
-        <v>218</v>
+        <v>169</v>
+      </c>
+      <c r="I239" s="3" t="n">
+        <v>245</v>
       </c>
     </row>
     <row r="240">
@@ -8192,7 +8911,10 @@
         <v>0</v>
       </c>
       <c r="H240" s="3" t="n">
-        <v>245</v>
+        <v>191</v>
+      </c>
+      <c r="I240" s="3" t="n">
+        <v>291</v>
       </c>
     </row>
     <row r="241">
@@ -8224,7 +8946,10 @@
         <v>0</v>
       </c>
       <c r="H241" s="3" t="n">
-        <v>220</v>
+        <v>168</v>
+      </c>
+      <c r="I241" s="3" t="n">
+        <v>249</v>
       </c>
     </row>
     <row r="242">
@@ -8256,7 +8981,10 @@
         <v>0</v>
       </c>
       <c r="H242" s="3" t="n">
-        <v>237</v>
+        <v>199</v>
+      </c>
+      <c r="I242" s="3" t="n">
+        <v>277</v>
       </c>
     </row>
     <row r="243">
@@ -8288,7 +9016,10 @@
         <v>0</v>
       </c>
       <c r="H243" s="3" t="n">
-        <v>180</v>
+        <v>252</v>
+      </c>
+      <c r="I243" s="3" t="n">
+        <v>207</v>
       </c>
     </row>
     <row r="244">
@@ -8320,7 +9051,10 @@
         <v>0</v>
       </c>
       <c r="H244" s="3" t="n">
-        <v>202</v>
+        <v>240</v>
+      </c>
+      <c r="I244" s="3" t="n">
+        <v>221</v>
       </c>
     </row>
     <row r="245">
@@ -8352,7 +9086,10 @@
         <v>0</v>
       </c>
       <c r="H245" s="3" t="n">
-        <v>212</v>
+        <v>176</v>
+      </c>
+      <c r="I245" s="3" t="n">
+        <v>240</v>
       </c>
     </row>
     <row r="246">
@@ -8384,7 +9121,10 @@
         <v>0</v>
       </c>
       <c r="H246" s="3" t="n">
-        <v>214</v>
+        <v>174</v>
+      </c>
+      <c r="I246" s="3" t="n">
+        <v>242</v>
       </c>
     </row>
     <row r="247">
@@ -8416,7 +9156,10 @@
         <v>0</v>
       </c>
       <c r="H247" s="3" t="n">
-        <v>195</v>
+        <v>246</v>
+      </c>
+      <c r="I247" s="3" t="n">
+        <v>212</v>
       </c>
     </row>
     <row r="248">
@@ -8448,7 +9191,10 @@
         <v>0</v>
       </c>
       <c r="H248" s="3" t="n">
-        <v>254</v>
+        <v>182</v>
+      </c>
+      <c r="I248" s="3" t="n">
+        <v>293</v>
       </c>
     </row>
     <row r="249">
@@ -8480,7 +9226,10 @@
         <v>0</v>
       </c>
       <c r="H249" s="3" t="n">
-        <v>221</v>
+        <v>166</v>
+      </c>
+      <c r="I249" s="3" t="n">
+        <v>264</v>
       </c>
     </row>
     <row r="250">
@@ -8512,7 +9261,10 @@
         <v>0</v>
       </c>
       <c r="H250" s="3" t="n">
-        <v>252</v>
+        <v>184</v>
+      </c>
+      <c r="I250" s="3" t="n">
+        <v>263</v>
       </c>
     </row>
     <row r="251">
@@ -8544,7 +9296,10 @@
         <v>0</v>
       </c>
       <c r="H251" s="3" t="n">
-        <v>249</v>
+        <v>187</v>
+      </c>
+      <c r="I251" s="3" t="n">
+        <v>292</v>
       </c>
     </row>
     <row r="252">
@@ -8578,6 +9333,9 @@
       <c r="H252" s="3" t="n">
         <v>255</v>
       </c>
+      <c r="I252" s="3" t="n">
+        <v>229</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="8" t="inlineStr">
@@ -8608,7 +9366,10 @@
         <v>0</v>
       </c>
       <c r="H253" s="3" t="n">
-        <v>225</v>
+        <v>163</v>
+      </c>
+      <c r="I253" s="3" t="n">
+        <v>261</v>
       </c>
     </row>
     <row r="254">
@@ -8640,7 +9401,10 @@
         <v>0</v>
       </c>
       <c r="H254" s="3" t="n">
-        <v>224</v>
+        <v>161</v>
+      </c>
+      <c r="I254" s="3" t="n">
+        <v>257</v>
       </c>
     </row>
     <row r="255">
@@ -8672,7 +9436,10 @@
         <v>0</v>
       </c>
       <c r="H255" s="3" t="n">
-        <v>234</v>
+        <v>202</v>
+      </c>
+      <c r="I255" s="3" t="n">
+        <v>256</v>
       </c>
     </row>
     <row r="256">
@@ -8704,7 +9471,10 @@
         <v>0</v>
       </c>
       <c r="H256" s="3" t="n">
-        <v>213</v>
+        <v>175</v>
+      </c>
+      <c r="I256" s="3" t="n">
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh ESPN and Yahoo adjusted rankings
</commit_message>
<xml_diff>
--- a/frontend/public/data/2026/espn/merged_formatted.xlsx
+++ b/frontend/public/data/2026/espn/merged_formatted.xlsx
@@ -616,7 +616,7 @@
         <v>55</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>4</v>
@@ -651,7 +651,7 @@
         <v>56</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>2</v>
@@ -791,7 +791,7 @@
         <v>51</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>6</v>
@@ -826,7 +826,7 @@
         <v>54</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>7</v>
@@ -1351,7 +1351,7 @@
         <v>21</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>36</v>
@@ -1386,7 +1386,7 @@
         <v>37</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>18</v>
@@ -1771,7 +1771,7 @@
         <v>30</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>26</v>
@@ -1806,7 +1806,7 @@
         <v>22</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>29</v>
@@ -1876,7 +1876,7 @@
         <v>22</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>38</v>
@@ -1911,7 +1911,7 @@
         <v>19</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>43</v>
@@ -2156,7 +2156,7 @@
         <v>26</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>31</v>
@@ -2191,7 +2191,7 @@
         <v>30</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>27</v>
@@ -2261,7 +2261,7 @@
         <v>19</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I50" s="3" t="n">
         <v>41</v>
@@ -2296,7 +2296,7 @@
         <v>9</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I51" s="3" t="n">
         <v>58</v>
@@ -2366,7 +2366,7 @@
         <v>12</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I53" s="3" t="n">
         <v>50</v>
@@ -2401,7 +2401,7 @@
         <v>15</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I54" s="3" t="n">
         <v>51</v>
@@ -2436,7 +2436,7 @@
         <v>15</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I55" s="3" t="n">
         <v>52</v>
@@ -2471,7 +2471,7 @@
         <v>8</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="I56" s="3" t="n">
         <v>59</v>
@@ -2506,7 +2506,7 @@
         <v>10</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I57" s="3" t="n">
         <v>45</v>
@@ -2541,7 +2541,7 @@
         <v>6</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I58" s="3" t="n">
         <v>61</v>
@@ -2576,7 +2576,7 @@
         <v>6</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I59" s="3" t="n">
         <v>62</v>
@@ -2611,7 +2611,7 @@
         <v>7</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I60" s="3" t="n">
         <v>72</v>
@@ -2646,7 +2646,7 @@
         <v>10</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I61" s="3" t="n">
         <v>57</v>
@@ -2681,7 +2681,7 @@
         <v>13</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I62" s="3" t="n">
         <v>49</v>
@@ -2751,7 +2751,7 @@
         <v>7</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I64" s="3" t="n">
         <v>63</v>
@@ -2786,7 +2786,7 @@
         <v>6</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I65" s="3" t="n">
         <v>71</v>
@@ -2821,7 +2821,7 @@
         <v>2</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I66" s="3" t="n">
         <v>108</v>
@@ -2856,7 +2856,7 @@
         <v>2</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I67" s="3" t="n">
         <v>109</v>
@@ -2926,7 +2926,7 @@
         <v>5</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I69" s="3" t="n">
         <v>75</v>
@@ -2961,7 +2961,7 @@
         <v>4</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I70" s="3" t="n">
         <v>84</v>
@@ -2996,7 +2996,7 @@
         <v>5</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="I71" s="3" t="n">
         <v>76</v>
@@ -3031,7 +3031,7 @@
         <v>6</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I72" s="3" t="n">
         <v>78</v>
@@ -3066,7 +3066,7 @@
         <v>4</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I73" s="3" t="n">
         <v>81</v>
@@ -3101,7 +3101,7 @@
         <v>4</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I74" s="3" t="n">
         <v>79</v>
@@ -3136,7 +3136,7 @@
         <v>8</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I75" s="3" t="n">
         <v>60</v>
@@ -3171,7 +3171,7 @@
         <v>2</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I76" s="3" t="n">
         <v>105</v>
@@ -3241,7 +3241,7 @@
         <v>10</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I78" s="3" t="n">
         <v>66</v>
@@ -3276,7 +3276,7 @@
         <v>14</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="I79" s="3" t="n">
         <v>47</v>
@@ -3311,7 +3311,7 @@
         <v>3</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I80" s="3" t="n">
         <v>100</v>
@@ -3416,7 +3416,7 @@
         <v>2</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I83" s="3" t="n">
         <v>97</v>
@@ -3451,7 +3451,7 @@
         <v>4</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="I84" s="3" t="n">
         <v>68</v>
@@ -3486,7 +3486,7 @@
         <v>2</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I85" s="3" t="n">
         <v>96</v>
@@ -3556,7 +3556,7 @@
         <v>2</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="I87" s="3" t="n">
         <v>98</v>
@@ -3591,7 +3591,7 @@
         <v>6</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I88" s="3" t="n">
         <v>67</v>
@@ -3626,7 +3626,7 @@
         <v>1</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I89" s="3" t="n">
         <v>149</v>
@@ -3661,7 +3661,7 @@
         <v>1</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I90" s="3" t="n">
         <v>136</v>
@@ -3696,7 +3696,7 @@
         <v>3</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I91" s="3" t="n">
         <v>91</v>
@@ -3731,7 +3731,7 @@
         <v>4</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="I92" s="3" t="n">
         <v>85</v>
@@ -3836,7 +3836,7 @@
         <v>2</v>
       </c>
       <c r="H95" s="3" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="I95" s="3" t="n">
         <v>118</v>
@@ -3871,7 +3871,7 @@
         <v>9</v>
       </c>
       <c r="H96" s="3" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I96" s="3" t="n">
         <v>64</v>
@@ -3906,7 +3906,7 @@
         <v>7</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="I97" s="3" t="n">
         <v>70</v>
@@ -3941,7 +3941,7 @@
         <v>2</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="I98" s="3" t="n">
         <v>111</v>
@@ -3976,7 +3976,7 @@
         <v>1</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I99" s="3" t="n">
         <v>137</v>
@@ -4011,7 +4011,7 @@
         <v>3</v>
       </c>
       <c r="H100" s="3" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I100" s="3" t="n">
         <v>86</v>
@@ -4046,7 +4046,7 @@
         <v>1</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I101" s="3" t="n">
         <v>138</v>
@@ -4081,7 +4081,7 @@
         <v>1</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="I102" s="3" t="n">
         <v>130</v>
@@ -4116,7 +4116,7 @@
         <v>4</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I103" s="3" t="n">
         <v>80</v>
@@ -4151,7 +4151,7 @@
         <v>2</v>
       </c>
       <c r="H104" s="3" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I104" s="3" t="n">
         <v>121</v>
@@ -4186,7 +4186,7 @@
         <v>1</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="I105" s="3" t="n">
         <v>131</v>
@@ -4221,7 +4221,7 @@
         <v>3</v>
       </c>
       <c r="H106" s="3" t="n">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="I106" s="3" t="n">
         <v>87</v>
@@ -4256,7 +4256,7 @@
         <v>2</v>
       </c>
       <c r="H107" s="3" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I107" s="3" t="n">
         <v>93</v>
@@ -4291,7 +4291,7 @@
         <v>3</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="I108" s="3" t="n">
         <v>82</v>
@@ -4326,7 +4326,7 @@
         <v>2</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="I109" s="3" t="n">
         <v>103</v>
@@ -4361,7 +4361,7 @@
         <v>1</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I110" s="3" t="n">
         <v>152</v>
@@ -4396,7 +4396,7 @@
         <v>2</v>
       </c>
       <c r="H111" s="3" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I111" s="3" t="n">
         <v>122</v>
@@ -4431,7 +4431,7 @@
         <v>0</v>
       </c>
       <c r="H112" s="3" t="n">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="I112" s="3" t="n">
         <v>217</v>
@@ -4466,7 +4466,7 @@
         <v>1</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I113" s="3" t="n">
         <v>148</v>
@@ -4501,7 +4501,7 @@
         <v>3</v>
       </c>
       <c r="H114" s="3" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I114" s="3" t="n">
         <v>102</v>
@@ -4536,7 +4536,7 @@
         <v>4</v>
       </c>
       <c r="H115" s="3" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="I115" s="3" t="n">
         <v>90</v>
@@ -4571,7 +4571,7 @@
         <v>2</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="I116" s="3" t="n">
         <v>95</v>
@@ -4606,7 +4606,7 @@
         <v>0</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="I117" s="3" t="n">
         <v>260</v>
@@ -4641,7 +4641,7 @@
         <v>2</v>
       </c>
       <c r="H118" s="3" t="n">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="I118" s="3" t="n">
         <v>129</v>
@@ -4676,7 +4676,7 @@
         <v>2</v>
       </c>
       <c r="H119" s="3" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="I119" s="3" t="n">
         <v>116</v>
@@ -4711,7 +4711,7 @@
         <v>1</v>
       </c>
       <c r="H120" s="3" t="n">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="I120" s="3" t="n">
         <v>183</v>
@@ -4746,7 +4746,7 @@
         <v>3</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I121" s="3" t="n">
         <v>88</v>
@@ -4781,7 +4781,7 @@
         <v>2</v>
       </c>
       <c r="H122" s="3" t="n">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="I122" s="3" t="n">
         <v>94</v>
@@ -4816,7 +4816,7 @@
         <v>1</v>
       </c>
       <c r="H123" s="3" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="I123" s="3" t="n">
         <v>147</v>
@@ -4886,7 +4886,7 @@
         <v>5</v>
       </c>
       <c r="H125" s="3" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I125" s="3" t="n">
         <v>83</v>
@@ -4921,7 +4921,7 @@
         <v>2</v>
       </c>
       <c r="H126" s="3" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I126" s="3" t="n">
         <v>125</v>
@@ -4956,7 +4956,7 @@
         <v>1</v>
       </c>
       <c r="H127" s="3" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I127" s="3" t="n">
         <v>150</v>
@@ -4971,30 +4971,30 @@
       <c r="B128" s="3" t="n">
         <v>127</v>
       </c>
-      <c r="C128" s="10" t="n">
-        <v>93</v>
+      <c r="C128" s="9" t="n">
+        <v>84</v>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Chris Godwin</t>
+          <t>Stefon Diggs</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>WAS</t>
         </is>
       </c>
       <c r="F128" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G128" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H128" s="3" t="n">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="I128" s="3" t="n">
-        <v>101</v>
+        <v>92</v>
       </c>
     </row>
     <row r="129">
@@ -5006,30 +5006,30 @@
       <c r="B129" s="3" t="n">
         <v>128</v>
       </c>
-      <c r="C129" s="4" t="n">
-        <v>134</v>
+      <c r="C129" s="10" t="n">
+        <v>93</v>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>Romeo Doubs</t>
+          <t>Chris Godwin</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="F129" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G129" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H129" s="3" t="n">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="I129" s="3" t="n">
-        <v>135</v>
+        <v>101</v>
       </c>
     </row>
     <row r="130">
@@ -5042,16 +5042,16 @@
         <v>129</v>
       </c>
       <c r="C130" s="4" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Jayden Higgins</t>
+          <t>Romeo Doubs</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="F130" s="3" t="n">
@@ -5061,10 +5061,10 @@
         <v>1</v>
       </c>
       <c r="H130" s="3" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="I130" s="3" t="n">
-        <v>124</v>
+        <v>135</v>
       </c>
     </row>
     <row r="131">
@@ -5077,29 +5077,29 @@
         <v>130</v>
       </c>
       <c r="C131" s="4" t="n">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>Jalen Coker</t>
+          <t>Jayden Higgins</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="F131" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G131" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H131" s="3" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I131" s="3" t="n">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="132">
@@ -5111,30 +5111,30 @@
       <c r="B132" s="3" t="n">
         <v>131</v>
       </c>
-      <c r="C132" s="7" t="n">
-        <v>191</v>
+      <c r="C132" s="4" t="n">
+        <v>119</v>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Jerry Jeudy</t>
+          <t>Jalen Coker</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="F132" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G132" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H132" s="3" t="n">
-        <v>147</v>
+        <v>127</v>
       </c>
       <c r="I132" s="3" t="n">
-        <v>198</v>
+        <v>110</v>
       </c>
     </row>
     <row r="133">
@@ -5146,30 +5146,30 @@
       <c r="B133" s="3" t="n">
         <v>132</v>
       </c>
-      <c r="C133" s="4" t="n">
-        <v>131</v>
+      <c r="C133" s="7" t="n">
+        <v>191</v>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>Rashid Shaheed</t>
+          <t>Jerry Jeudy</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="F133" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G133" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H133" s="3" t="n">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="I133" s="3" t="n">
-        <v>134</v>
+        <v>198</v>
       </c>
     </row>
     <row r="134">
@@ -5201,7 +5201,7 @@
         <v>1</v>
       </c>
       <c r="H134" s="3" t="n">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="I134" s="3" t="n">
         <v>120</v>
@@ -5236,7 +5236,7 @@
         <v>0</v>
       </c>
       <c r="H135" s="3" t="n">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="I135" s="3" t="n">
         <v>166</v>
@@ -5271,7 +5271,7 @@
         <v>2</v>
       </c>
       <c r="H136" s="3" t="n">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="I136" s="3" t="n">
         <v>114</v>
@@ -5306,7 +5306,7 @@
         <v>0</v>
       </c>
       <c r="H137" s="3" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I137" s="3" t="n">
         <v>178</v>
@@ -5341,7 +5341,7 @@
         <v>2</v>
       </c>
       <c r="H138" s="3" t="n">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="I138" s="3" t="n">
         <v>104</v>
@@ -5376,7 +5376,7 @@
         <v>0</v>
       </c>
       <c r="H139" s="3" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="I139" s="3" t="n">
         <v>186</v>
@@ -5411,7 +5411,7 @@
         <v>0</v>
       </c>
       <c r="H140" s="3" t="n">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="I140" s="3" t="n">
         <v>171</v>
@@ -5481,7 +5481,7 @@
         <v>0</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="I142" s="3" t="n">
         <v>170</v>
@@ -5516,7 +5516,7 @@
         <v>0</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="I143" s="3" t="n">
         <v>156</v>
@@ -5531,30 +5531,30 @@
       <c r="B144" s="3" t="n">
         <v>143</v>
       </c>
-      <c r="C144" s="7" t="n">
-        <v>172</v>
+      <c r="C144" s="4" t="n">
+        <v>131</v>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Jalen McMillan</t>
+          <t>Rashid Shaheed</t>
         </is>
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="F144" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G144" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H144" s="3" t="n">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="I144" s="3" t="n">
-        <v>158</v>
+        <v>134</v>
       </c>
     </row>
     <row r="145">
@@ -5567,16 +5567,16 @@
         <v>144</v>
       </c>
       <c r="C145" s="7" t="n">
-        <v>231</v>
+        <v>172</v>
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>Calvin Ridley</t>
+          <t>Jalen McMillan</t>
         </is>
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="F145" s="3" t="n">
@@ -5589,7 +5589,7 @@
         <v>155</v>
       </c>
       <c r="I145" s="3" t="n">
-        <v>216</v>
+        <v>158</v>
       </c>
     </row>
     <row r="146">
@@ -5601,30 +5601,30 @@
       <c r="B146" s="3" t="n">
         <v>145</v>
       </c>
-      <c r="C146" s="4" t="n">
-        <v>146</v>
+      <c r="C146" s="7" t="n">
+        <v>231</v>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Denzel Boston</t>
+          <t>Calvin Ridley</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="F146" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G146" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="I146" s="3" t="n">
-        <v>181</v>
+        <v>216</v>
       </c>
     </row>
     <row r="147">
@@ -5636,17 +5636,17 @@
       <c r="B147" s="3" t="n">
         <v>146</v>
       </c>
-      <c r="C147" s="5" t="n">
-        <v>158</v>
+      <c r="C147" s="4" t="n">
+        <v>146</v>
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>Travis Hunter</t>
+          <t>Denzel Boston</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
         <is>
-          <t>JAC</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="F147" s="3" t="n">
@@ -5656,10 +5656,10 @@
         <v>1</v>
       </c>
       <c r="H147" s="3" t="n">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="I147" s="3" t="n">
-        <v>151</v>
+        <v>181</v>
       </c>
     </row>
     <row r="148">
@@ -5671,30 +5671,30 @@
       <c r="B148" s="3" t="n">
         <v>147</v>
       </c>
-      <c r="C148" s="7" t="n">
-        <v>190</v>
+      <c r="C148" s="5" t="n">
+        <v>158</v>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Adonai Mitchell</t>
+          <t>Travis Hunter</t>
         </is>
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>NYJ</t>
+          <t>JAC</t>
         </is>
       </c>
       <c r="F148" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G148" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H148" s="3" t="n">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="I148" s="3" t="n">
-        <v>197</v>
+        <v>151</v>
       </c>
     </row>
     <row r="149">
@@ -5706,30 +5706,30 @@
       <c r="B149" s="3" t="n">
         <v>148</v>
       </c>
-      <c r="C149" s="4" t="n">
-        <v>129</v>
+      <c r="C149" s="7" t="n">
+        <v>190</v>
       </c>
       <c r="D149" s="3" t="inlineStr">
         <is>
-          <t>De'Zhaun Stribling</t>
+          <t>Adonai Mitchell</t>
         </is>
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>NYJ</t>
         </is>
       </c>
       <c r="F149" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G149" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="I149" s="3" t="n">
-        <v>126</v>
+        <v>197</v>
       </c>
     </row>
     <row r="150">
@@ -5761,7 +5761,7 @@
         <v>1</v>
       </c>
       <c r="H150" s="3" t="n">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="I150" s="3" t="n">
         <v>119</v>
@@ -5796,7 +5796,7 @@
         <v>1</v>
       </c>
       <c r="H151" s="3" t="n">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="I151" s="3" t="n">
         <v>133</v>
@@ -5811,30 +5811,30 @@
       <c r="B152" s="3" t="n">
         <v>151</v>
       </c>
-      <c r="C152" s="5" t="n">
-        <v>255</v>
+      <c r="C152" s="4" t="n">
+        <v>129</v>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Germie Bernard</t>
+          <t>De'Zhaun Stribling</t>
         </is>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="F152" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G152" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="I152" s="3" t="n">
-        <v>223</v>
+        <v>126</v>
       </c>
     </row>
     <row r="153">
@@ -5847,16 +5847,16 @@
         <v>152</v>
       </c>
       <c r="C153" s="5" t="n">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="D153" s="3" t="inlineStr">
         <is>
-          <t>Antonio Williams</t>
+          <t>Germie Bernard</t>
         </is>
       </c>
       <c r="E153" s="3" t="inlineStr">
         <is>
-          <t>WAS</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="F153" s="3" t="n">
@@ -5866,10 +5866,10 @@
         <v>0</v>
       </c>
       <c r="H153" s="3" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I153" s="3" t="n">
-        <v>268</v>
+        <v>223</v>
       </c>
     </row>
     <row r="154">
@@ -5901,7 +5901,7 @@
         <v>0</v>
       </c>
       <c r="H154" s="3" t="n">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="I154" s="3" t="n">
         <v>213</v>
@@ -5936,7 +5936,7 @@
         <v>0</v>
       </c>
       <c r="H155" s="3" t="n">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="I155" s="3" t="n">
         <v>192</v>
@@ -5971,7 +5971,7 @@
         <v>1</v>
       </c>
       <c r="H156" s="3" t="n">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="I156" s="3" t="n">
         <v>155</v>
@@ -6006,7 +6006,7 @@
         <v>0</v>
       </c>
       <c r="H157" s="3" t="n">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="I157" s="3" t="n">
         <v>209</v>
@@ -6041,7 +6041,7 @@
         <v>0</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="I158" s="3" t="n">
         <v>169</v>
@@ -6076,7 +6076,7 @@
         <v>0</v>
       </c>
       <c r="H159" s="3" t="n">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="I159" s="3" t="n">
         <v>194</v>
@@ -6111,7 +6111,7 @@
         <v>0</v>
       </c>
       <c r="H160" s="3" t="n">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="I160" s="3" t="n">
         <v>235</v>
@@ -6146,7 +6146,7 @@
         <v>1</v>
       </c>
       <c r="H161" s="3" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I161" s="3" t="n">
         <v>172</v>
@@ -6181,7 +6181,7 @@
         <v>1</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="I162" s="3" t="n">
         <v>157</v>
@@ -6216,7 +6216,7 @@
         <v>0</v>
       </c>
       <c r="H163" s="3" t="n">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="I163" s="3" t="n">
         <v>199</v>
@@ -6251,7 +6251,7 @@
         <v>0</v>
       </c>
       <c r="H164" s="3" t="n">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="I164" s="3" t="n">
         <v>215</v>
@@ -6286,7 +6286,7 @@
         <v>0</v>
       </c>
       <c r="H165" s="3" t="n">
-        <v>220</v>
+        <v>202</v>
       </c>
       <c r="I165" s="3" t="n">
         <v>200</v>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="H166" s="3" t="n">
-        <v>185</v>
+        <v>244</v>
       </c>
       <c r="I166" s="3" t="n">
         <v>262</v>
@@ -6356,7 +6356,7 @@
         <v>0</v>
       </c>
       <c r="H167" s="3" t="n">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="I167" s="3" t="n">
         <v>195</v>
@@ -6391,7 +6391,7 @@
         <v>0</v>
       </c>
       <c r="H168" s="3" t="n">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="I168" s="3" t="n">
         <v>225</v>
@@ -6426,7 +6426,7 @@
         <v>2</v>
       </c>
       <c r="H169" s="3" t="n">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="I169" s="3" t="n">
         <v>123</v>
@@ -6461,7 +6461,7 @@
         <v>2</v>
       </c>
       <c r="H170" s="3" t="n">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="I170" s="3" t="n">
         <v>107</v>
@@ -6496,7 +6496,7 @@
         <v>1</v>
       </c>
       <c r="H171" s="3" t="n">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="I171" s="3" t="n">
         <v>140</v>
@@ -6531,7 +6531,7 @@
         <v>0</v>
       </c>
       <c r="H172" s="3" t="n">
-        <v>204</v>
+        <v>183</v>
       </c>
       <c r="I172" s="3" t="n">
         <v>153</v>
@@ -6566,7 +6566,7 @@
         <v>0</v>
       </c>
       <c r="H173" s="3" t="n">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="I173" s="3" t="n">
         <v>164</v>
@@ -6601,7 +6601,7 @@
         <v>1</v>
       </c>
       <c r="H174" s="3" t="n">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="I174" s="3" t="n">
         <v>141</v>
@@ -6636,7 +6636,7 @@
         <v>0</v>
       </c>
       <c r="H175" s="3" t="n">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="I175" s="3" t="n">
         <v>163</v>
@@ -6671,7 +6671,7 @@
         <v>0</v>
       </c>
       <c r="H176" s="3" t="n">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="I176" s="3" t="n">
         <v>202</v>
@@ -6706,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="H177" s="3" t="n">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="I177" s="3" t="n">
         <v>139</v>
@@ -6741,7 +6741,7 @@
         <v>1</v>
       </c>
       <c r="H178" s="3" t="n">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="I178" s="3" t="n">
         <v>145</v>
@@ -6776,7 +6776,7 @@
         <v>0</v>
       </c>
       <c r="H179" s="3" t="n">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="I179" s="3" t="n">
         <v>162</v>
@@ -6811,7 +6811,7 @@
         <v>0</v>
       </c>
       <c r="H180" s="3" t="n">
-        <v>205</v>
+        <v>184</v>
       </c>
       <c r="I180" s="3" t="n">
         <v>161</v>
@@ -6846,7 +6846,7 @@
         <v>0</v>
       </c>
       <c r="H181" s="3" t="n">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="I181" s="3" t="n">
         <v>228</v>
@@ -6881,7 +6881,7 @@
         <v>0</v>
       </c>
       <c r="H182" s="3" t="n">
-        <v>166</v>
+        <v>257</v>
       </c>
       <c r="I182" s="3" t="n">
         <v>253</v>
@@ -6916,7 +6916,7 @@
         <v>0</v>
       </c>
       <c r="H183" s="3" t="n">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="I183" s="3" t="n">
         <v>185</v>
@@ -6951,7 +6951,7 @@
         <v>0</v>
       </c>
       <c r="H184" s="3" t="n">
-        <v>163</v>
+        <v>253</v>
       </c>
       <c r="I184" s="3" t="n">
         <v>243</v>
@@ -6986,7 +6986,7 @@
         <v>0</v>
       </c>
       <c r="H185" s="3" t="n">
-        <v>243</v>
+        <v>227</v>
       </c>
       <c r="I185" s="3" t="n">
         <v>239</v>
@@ -7021,7 +7021,7 @@
         <v>0</v>
       </c>
       <c r="H186" s="3" t="n">
-        <v>256</v>
+        <v>241</v>
       </c>
       <c r="I186" s="3" t="n">
         <v>250</v>
@@ -7056,7 +7056,7 @@
         <v>2</v>
       </c>
       <c r="H187" s="3" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I187" s="3" t="n">
         <v>115</v>
@@ -7091,7 +7091,7 @@
         <v>0</v>
       </c>
       <c r="H188" s="3" t="n">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="I188" s="3" t="n">
         <v>206</v>
@@ -7126,7 +7126,7 @@
         <v>0</v>
       </c>
       <c r="H189" s="3" t="n">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="I189" s="3" t="n">
         <v>165</v>
@@ -7161,7 +7161,7 @@
         <v>0</v>
       </c>
       <c r="H190" s="3" t="n">
-        <v>178</v>
+        <v>272</v>
       </c>
       <c r="I190" s="3" t="n">
         <v>274</v>
@@ -7174,32 +7174,32 @@
         </is>
       </c>
       <c r="B191" s="3" t="n">
-        <v>202</v>
-      </c>
-      <c r="C191" s="9" t="n">
-        <v>84</v>
+        <v>203</v>
+      </c>
+      <c r="C191" s="10" t="n">
+        <v>171</v>
       </c>
       <c r="D191" s="3" t="inlineStr">
         <is>
-          <t>Stefon Diggs</t>
+          <t>Ryan Flournoy</t>
         </is>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>WAS</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="F191" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G191" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H191" s="3" t="n">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="I191" s="3" t="n">
-        <v>92</v>
+        <v>180</v>
       </c>
     </row>
     <row r="192">
@@ -7211,17 +7211,17 @@
       <c r="B192" s="3" t="n">
         <v>204</v>
       </c>
-      <c r="C192" s="10" t="n">
-        <v>171</v>
+      <c r="C192" s="5" t="n">
+        <v>268</v>
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>Ryan Flournoy</t>
+          <t>Antonio Williams</t>
         </is>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>WAS</t>
         </is>
       </c>
       <c r="F192" s="3" t="n">
@@ -7231,10 +7231,10 @@
         <v>0</v>
       </c>
       <c r="H192" s="3" t="n">
-        <v>217</v>
+        <v>250</v>
       </c>
       <c r="I192" s="3" t="n">
-        <v>180</v>
+        <v>268</v>
       </c>
     </row>
     <row r="193">
@@ -7266,7 +7266,7 @@
         <v>0</v>
       </c>
       <c r="H193" s="3" t="n">
-        <v>183</v>
+        <v>269</v>
       </c>
       <c r="I193" s="3" t="n">
         <v>275</v>
@@ -7301,7 +7301,7 @@
         <v>0</v>
       </c>
       <c r="H194" s="3" t="n">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="I194" s="3" t="n">
         <v>272</v>
@@ -7336,7 +7336,7 @@
         <v>0</v>
       </c>
       <c r="H195" s="3" t="n">
-        <v>226</v>
+        <v>210</v>
       </c>
       <c r="I195" s="3" t="n">
         <v>219</v>
@@ -7371,7 +7371,7 @@
         <v>0</v>
       </c>
       <c r="H196" s="3" t="n">
-        <v>262</v>
+        <v>166</v>
       </c>
       <c r="I196" s="3" t="inlineStr"/>
     </row>
@@ -7404,7 +7404,7 @@
         <v>0</v>
       </c>
       <c r="H197" s="3" t="n">
-        <v>189</v>
+        <v>246</v>
       </c>
       <c r="I197" s="3" t="n">
         <v>244</v>
@@ -7439,7 +7439,7 @@
         <v>0</v>
       </c>
       <c r="H198" s="3" t="n">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="I198" s="3" t="n">
         <v>214</v>
@@ -7474,7 +7474,7 @@
         <v>0</v>
       </c>
       <c r="H199" s="3" t="n">
-        <v>181</v>
+        <v>268</v>
       </c>
       <c r="I199" s="3" t="n">
         <v>269</v>
@@ -7509,7 +7509,7 @@
         <v>0</v>
       </c>
       <c r="H200" s="3" t="n">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="I200" s="3" t="n">
         <v>210</v>
@@ -7544,7 +7544,7 @@
         <v>0</v>
       </c>
       <c r="H201" s="3" t="n">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="I201" s="3" t="n">
         <v>211</v>
@@ -7579,7 +7579,7 @@
         <v>0</v>
       </c>
       <c r="H202" s="3" t="n">
-        <v>248</v>
+        <v>232</v>
       </c>
       <c r="I202" s="3" t="n">
         <v>224</v>
@@ -7614,7 +7614,7 @@
         <v>0</v>
       </c>
       <c r="H203" s="3" t="n">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="I203" s="3" t="n">
         <v>236</v>
@@ -7649,7 +7649,7 @@
         <v>1</v>
       </c>
       <c r="H204" s="3" t="n">
-        <v>208</v>
+        <v>185</v>
       </c>
       <c r="I204" s="3" t="n">
         <v>173</v>
@@ -7684,7 +7684,7 @@
         <v>0</v>
       </c>
       <c r="H205" s="3" t="n">
-        <v>215</v>
+        <v>190</v>
       </c>
       <c r="I205" s="3" t="n">
         <v>184</v>
@@ -7719,7 +7719,7 @@
         <v>0</v>
       </c>
       <c r="H206" s="3" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="I206" s="3" t="n">
         <v>167</v>
@@ -7754,7 +7754,7 @@
         <v>0</v>
       </c>
       <c r="H207" s="3" t="n">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="I207" s="3" t="n">
         <v>177</v>
@@ -7789,7 +7789,7 @@
         <v>0</v>
       </c>
       <c r="H208" s="3" t="n">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="I208" s="3" t="n">
         <v>208</v>
@@ -7824,7 +7824,7 @@
         <v>0</v>
       </c>
       <c r="H209" s="3" t="n">
-        <v>174</v>
+        <v>264</v>
       </c>
       <c r="I209" s="3" t="n">
         <v>279</v>
@@ -7840,7 +7840,7 @@
         <v>222</v>
       </c>
       <c r="C210" s="5" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
@@ -7859,7 +7859,7 @@
         <v>0</v>
       </c>
       <c r="H210" s="3" t="n">
-        <v>190</v>
+        <v>245</v>
       </c>
       <c r="I210" s="3" t="n">
         <v>287</v>
@@ -7894,7 +7894,7 @@
         <v>0</v>
       </c>
       <c r="H211" s="3" t="n">
-        <v>169</v>
+        <v>259</v>
       </c>
       <c r="I211" s="3" t="n">
         <v>252</v>
@@ -7929,7 +7929,7 @@
         <v>0</v>
       </c>
       <c r="H212" s="3" t="n">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="I212" s="3" t="n">
         <v>196</v>
@@ -7964,7 +7964,7 @@
         <v>0</v>
       </c>
       <c r="H213" s="3" t="n">
-        <v>179</v>
+        <v>271</v>
       </c>
       <c r="I213" s="3" t="n">
         <v>280</v>
@@ -7999,7 +7999,7 @@
         <v>0</v>
       </c>
       <c r="H214" s="3" t="n">
-        <v>229</v>
+        <v>216</v>
       </c>
       <c r="I214" s="3" t="n">
         <v>281</v>
@@ -8034,7 +8034,7 @@
         <v>0</v>
       </c>
       <c r="H215" s="3" t="n">
-        <v>175</v>
+        <v>265</v>
       </c>
       <c r="I215" s="3" t="n">
         <v>278</v>
@@ -8069,7 +8069,7 @@
         <v>0</v>
       </c>
       <c r="H216" s="3" t="n">
-        <v>187</v>
+        <v>248</v>
       </c>
       <c r="I216" s="3" t="n">
         <v>237</v>
@@ -8104,7 +8104,7 @@
         <v>0</v>
       </c>
       <c r="H217" s="3" t="n">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="I217" s="3" t="n">
         <v>222</v>
@@ -8139,7 +8139,7 @@
         <v>0</v>
       </c>
       <c r="H218" s="3" t="n">
-        <v>191</v>
+        <v>256</v>
       </c>
       <c r="I218" s="3" t="n">
         <v>238</v>
@@ -8174,7 +8174,7 @@
         <v>0</v>
       </c>
       <c r="H219" s="3" t="n">
-        <v>192</v>
+        <v>242</v>
       </c>
       <c r="I219" s="3" t="n">
         <v>248</v>
@@ -8209,7 +8209,7 @@
         <v>0</v>
       </c>
       <c r="H220" s="3" t="n">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="I220" s="3" t="n">
         <v>246</v>
@@ -8244,7 +8244,7 @@
         <v>0</v>
       </c>
       <c r="H221" s="3" t="n">
-        <v>261</v>
+        <v>165</v>
       </c>
       <c r="I221" s="3" t="n">
         <v>283</v>
@@ -8279,7 +8279,7 @@
         <v>0</v>
       </c>
       <c r="H222" s="3" t="n">
-        <v>168</v>
+        <v>254</v>
       </c>
       <c r="I222" s="3" t="n">
         <v>288</v>
@@ -8314,7 +8314,7 @@
         <v>0</v>
       </c>
       <c r="H223" s="3" t="n">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="I223" s="3" t="n">
         <v>201</v>
@@ -8349,7 +8349,7 @@
         <v>0</v>
       </c>
       <c r="H224" s="3" t="n">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="I224" s="3" t="n">
         <v>187</v>
@@ -8365,7 +8365,7 @@
         <v>239</v>
       </c>
       <c r="C225" s="5" t="n">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D225" s="3" t="inlineStr">
         <is>
@@ -8384,7 +8384,7 @@
         <v>0</v>
       </c>
       <c r="H225" s="3" t="n">
-        <v>257</v>
+        <v>163</v>
       </c>
       <c r="I225" s="3" t="inlineStr"/>
     </row>
@@ -8417,7 +8417,7 @@
         <v>0</v>
       </c>
       <c r="H226" s="3" t="n">
-        <v>267</v>
+        <v>170</v>
       </c>
       <c r="I226" s="3" t="n">
         <v>285</v>
@@ -8452,7 +8452,7 @@
         <v>0</v>
       </c>
       <c r="H227" s="3" t="n">
-        <v>172</v>
+        <v>262</v>
       </c>
       <c r="I227" s="3" t="n">
         <v>286</v>
@@ -8487,7 +8487,7 @@
         <v>0</v>
       </c>
       <c r="H228" s="3" t="n">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="I228" s="3" t="n">
         <v>168</v>
@@ -8522,7 +8522,7 @@
         <v>0</v>
       </c>
       <c r="H229" s="3" t="n">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="I229" s="3" t="n">
         <v>193</v>
@@ -8557,7 +8557,7 @@
         <v>0</v>
       </c>
       <c r="H230" s="3" t="n">
-        <v>173</v>
+        <v>263</v>
       </c>
       <c r="I230" s="3" t="n">
         <v>276</v>
@@ -8592,7 +8592,7 @@
         <v>0</v>
       </c>
       <c r="H231" s="3" t="n">
-        <v>182</v>
+        <v>267</v>
       </c>
       <c r="I231" s="3" t="inlineStr"/>
     </row>
@@ -8625,7 +8625,7 @@
         <v>0</v>
       </c>
       <c r="H232" s="3" t="n">
-        <v>167</v>
+        <v>258</v>
       </c>
       <c r="I232" s="3" t="n">
         <v>266</v>
@@ -8660,7 +8660,7 @@
         <v>0</v>
       </c>
       <c r="H233" s="3" t="n">
-        <v>176</v>
+        <v>266</v>
       </c>
       <c r="I233" s="3" t="n">
         <v>289</v>
@@ -8695,7 +8695,7 @@
         <v>0</v>
       </c>
       <c r="H234" s="3" t="n">
-        <v>165</v>
+        <v>255</v>
       </c>
       <c r="I234" s="3" t="n">
         <v>265</v>
@@ -8730,7 +8730,7 @@
         <v>0</v>
       </c>
       <c r="H235" s="3" t="n">
-        <v>260</v>
+        <v>162</v>
       </c>
       <c r="I235" s="3" t="n">
         <v>290</v>
@@ -8765,7 +8765,7 @@
         <v>0</v>
       </c>
       <c r="H236" s="3" t="n">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="I236" s="3" t="n">
         <v>191</v>
@@ -8800,7 +8800,7 @@
         <v>0</v>
       </c>
       <c r="H237" s="3" t="n">
-        <v>164</v>
+        <v>252</v>
       </c>
       <c r="I237" s="3" t="n">
         <v>273</v>
@@ -8835,7 +8835,7 @@
         <v>0</v>
       </c>
       <c r="H238" s="3" t="n">
-        <v>218</v>
+        <v>191</v>
       </c>
       <c r="I238" s="3" t="n">
         <v>179</v>
@@ -8870,7 +8870,7 @@
         <v>0</v>
       </c>
       <c r="H239" s="3" t="n">
-        <v>271</v>
+        <v>174</v>
       </c>
       <c r="I239" s="3" t="inlineStr"/>
     </row>
@@ -8903,7 +8903,7 @@
         <v>1</v>
       </c>
       <c r="H240" s="3" t="n">
-        <v>198</v>
+        <v>182</v>
       </c>
       <c r="I240" s="3" t="n">
         <v>146</v>
@@ -8938,7 +8938,7 @@
         <v>0</v>
       </c>
       <c r="H241" s="3" t="n">
-        <v>249</v>
+        <v>233</v>
       </c>
       <c r="I241" s="3" t="inlineStr"/>
     </row>
@@ -8971,7 +8971,7 @@
         <v>0</v>
       </c>
       <c r="H242" s="3" t="n">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="I242" s="3" t="n">
         <v>220</v>
@@ -9006,7 +9006,7 @@
         <v>0</v>
       </c>
       <c r="H243" s="3" t="n">
-        <v>222</v>
+        <v>198</v>
       </c>
       <c r="I243" s="3" t="n">
         <v>218</v>
@@ -9041,7 +9041,7 @@
         <v>0</v>
       </c>
       <c r="H244" s="3" t="n">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="I244" s="3" t="n">
         <v>227</v>
@@ -9076,7 +9076,7 @@
         <v>0</v>
       </c>
       <c r="H245" s="3" t="n">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="I245" s="3" t="n">
         <v>245</v>
@@ -9111,7 +9111,7 @@
         <v>0</v>
       </c>
       <c r="H246" s="3" t="n">
-        <v>162</v>
+        <v>251</v>
       </c>
       <c r="I246" s="3" t="n">
         <v>291</v>
@@ -9146,7 +9146,7 @@
         <v>0</v>
       </c>
       <c r="H247" s="3" t="n">
-        <v>186</v>
+        <v>243</v>
       </c>
       <c r="I247" s="3" t="n">
         <v>249</v>
@@ -9181,7 +9181,7 @@
         <v>0</v>
       </c>
       <c r="H248" s="3" t="n">
-        <v>269</v>
+        <v>176</v>
       </c>
       <c r="I248" s="3" t="inlineStr"/>
     </row>
@@ -9214,7 +9214,7 @@
         <v>0</v>
       </c>
       <c r="H249" s="3" t="n">
-        <v>258</v>
+        <v>164</v>
       </c>
       <c r="I249" s="3" t="n">
         <v>277</v>
@@ -9249,7 +9249,7 @@
         <v>0</v>
       </c>
       <c r="H250" s="3" t="n">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="I250" s="3" t="n">
         <v>207</v>
@@ -9284,7 +9284,7 @@
         <v>0</v>
       </c>
       <c r="H251" s="3" t="n">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="I251" s="3" t="n">
         <v>221</v>
@@ -9319,7 +9319,7 @@
         <v>0</v>
       </c>
       <c r="H252" s="3" t="n">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="I252" s="3" t="n">
         <v>240</v>
@@ -9354,7 +9354,7 @@
         <v>0</v>
       </c>
       <c r="H253" s="3" t="n">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="I253" s="3" t="n">
         <v>242</v>
@@ -9389,7 +9389,7 @@
         <v>0</v>
       </c>
       <c r="H254" s="3" t="n">
-        <v>221</v>
+        <v>201</v>
       </c>
       <c r="I254" s="3" t="n">
         <v>212</v>
@@ -9424,7 +9424,7 @@
         <v>0</v>
       </c>
       <c r="H255" s="3" t="n">
-        <v>264</v>
+        <v>168</v>
       </c>
       <c r="I255" s="3" t="n">
         <v>293</v>
@@ -9459,7 +9459,7 @@
         <v>0</v>
       </c>
       <c r="H256" s="3" t="n">
-        <v>171</v>
+        <v>261</v>
       </c>
       <c r="I256" s="3" t="n">
         <v>264</v>
@@ -9494,7 +9494,7 @@
         <v>0</v>
       </c>
       <c r="H257" s="3" t="n">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="I257" s="3" t="n">
         <v>263</v>
@@ -9510,7 +9510,7 @@
         <v>275</v>
       </c>
       <c r="C258" s="4" t="n">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
@@ -9529,7 +9529,7 @@
         <v>0</v>
       </c>
       <c r="H258" s="3" t="n">
-        <v>188</v>
+        <v>247</v>
       </c>
       <c r="I258" s="3" t="inlineStr"/>
     </row>
@@ -9562,7 +9562,7 @@
         <v>0</v>
       </c>
       <c r="H259" s="3" t="n">
-        <v>161</v>
+        <v>249</v>
       </c>
       <c r="I259" s="3" t="inlineStr"/>
     </row>
@@ -9576,7 +9576,7 @@
         <v>279</v>
       </c>
       <c r="C260" s="4" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D260" s="3" t="inlineStr">
         <is>
@@ -9595,7 +9595,7 @@
         <v>0</v>
       </c>
       <c r="H260" s="3" t="n">
-        <v>259</v>
+        <v>161</v>
       </c>
       <c r="I260" s="3" t="inlineStr"/>
     </row>
@@ -9628,7 +9628,7 @@
         <v>0</v>
       </c>
       <c r="H261" s="3" t="n">
-        <v>266</v>
+        <v>171</v>
       </c>
       <c r="I261" s="3" t="inlineStr"/>
     </row>
@@ -9661,7 +9661,7 @@
         <v>0</v>
       </c>
       <c r="H262" s="3" t="n">
-        <v>263</v>
+        <v>167</v>
       </c>
       <c r="I262" s="3" t="inlineStr"/>
     </row>
@@ -9694,7 +9694,7 @@
         <v>0</v>
       </c>
       <c r="H263" s="3" t="n">
-        <v>265</v>
+        <v>172</v>
       </c>
       <c r="I263" s="3" t="inlineStr"/>
     </row>
@@ -9727,7 +9727,7 @@
         <v>0</v>
       </c>
       <c r="H264" s="3" t="n">
-        <v>270</v>
+        <v>175</v>
       </c>
       <c r="I264" s="3" t="inlineStr"/>
     </row>
@@ -9760,7 +9760,7 @@
         <v>0</v>
       </c>
       <c r="H265" s="3" t="n">
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="I265" s="3" t="n">
         <v>292</v>
@@ -9795,7 +9795,7 @@
         <v>0</v>
       </c>
       <c r="H266" s="3" t="n">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="I266" s="3" t="inlineStr"/>
     </row>
@@ -9828,7 +9828,7 @@
         <v>0</v>
       </c>
       <c r="H267" s="3" t="n">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="I267" s="3" t="n">
         <v>229</v>
@@ -9863,7 +9863,7 @@
         <v>0</v>
       </c>
       <c r="H268" s="3" t="n">
-        <v>170</v>
+        <v>260</v>
       </c>
       <c r="I268" s="3" t="n">
         <v>261</v>
@@ -9898,7 +9898,7 @@
         <v>0</v>
       </c>
       <c r="H269" s="3" t="n">
-        <v>253</v>
+        <v>237</v>
       </c>
       <c r="I269" s="3" t="n">
         <v>257</v>
@@ -9933,7 +9933,7 @@
         <v>0</v>
       </c>
       <c r="H270" s="3" t="n">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="I270" s="3" t="n">
         <v>256</v>
@@ -9968,7 +9968,7 @@
         <v>0</v>
       </c>
       <c r="H271" s="3" t="n">
-        <v>272</v>
+        <v>173</v>
       </c>
       <c r="I271" s="3" t="inlineStr"/>
     </row>
@@ -10001,7 +10001,7 @@
         <v>0</v>
       </c>
       <c r="H272" s="3" t="n">
-        <v>268</v>
+        <v>169</v>
       </c>
       <c r="I272" s="3" t="inlineStr"/>
     </row>
@@ -10034,7 +10034,7 @@
         <v>0</v>
       </c>
       <c r="H273" s="3" t="n">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="I273" s="3" t="n">
         <v>241</v>

</xml_diff>